<commit_message>
Updated Excel: merged Pasalubong into DAIKOKU DRUG, fixed names
</commit_message>
<xml_diff>
--- a/JAPAN EXPENSE.xlsx
+++ b/JAPAN EXPENSE.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d860ed5a51cbaf4b/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amadeusworkplace-my.sharepoint.com/personal/jonjester_reguyal_amadeus_com/Documents/Desktop/JAPAN TRIP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="303" documentId="8_{8DD0C82D-92A8-469F-8A5F-7373CA3C28E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8BD9314-1CB1-4FF9-93C2-9CBEA092C114}"/>
+  <xr:revisionPtr revIDLastSave="315" documentId="8_{8DD0C82D-92A8-469F-8A5F-7373CA3C28E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06E28EDE-50CA-4AE2-8124-1A3F23CBDC29}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{77262E9F-01AC-4670-AAC1-0C05B2A698AE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{77262E9F-01AC-4670-AAC1-0C05B2A698AE}"/>
   </bookViews>
   <sheets>
     <sheet name="Japan Trip" sheetId="1" r:id="rId1"/>
@@ -500,15 +500,6 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -521,6 +512,37 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -535,28 +557,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="2" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -897,7 +897,7 @@
   <dimension ref="B1:W96"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="8.88671875" style="23"/>
+    <col min="2" max="2" width="8.88671875" style="11"/>
     <col min="3" max="3" width="31.109375" customWidth="1"/>
     <col min="4" max="5" width="10.44140625" style="1" customWidth="1"/>
     <col min="6" max="10" width="8.88671875" hidden="1" customWidth="1"/>
@@ -911,70 +911,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
-      <c r="K1" s="24" t="s">
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="L1" s="24" t="s">
+      <c r="L1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="24" t="s">
+      <c r="M1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="N1" s="24" t="s">
+      <c r="N1" s="12" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B2" s="14">
+      <c r="B2" s="22">
         <v>42491</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
-      <c r="K2" s="10">
+      <c r="K2" s="7">
         <f>D3/2</f>
         <v>14785.36</v>
       </c>
-      <c r="L2" s="10">
+      <c r="L2" s="7">
         <f>D3/2</f>
         <v>14785.36</v>
       </c>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
     </row>
     <row r="3" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B3" s="14"/>
-      <c r="C3" s="11" t="s">
+      <c r="B3" s="22"/>
+      <c r="C3" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="7">
         <v>29570.720000000001</v>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="7">
         <f>SUM(D3)</f>
         <v>29570.720000000001</v>
       </c>
@@ -983,44 +983,44 @@
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
     </row>
     <row r="4" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B4" s="14"/>
+      <c r="B4" s="22"/>
       <c r="C4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
-      <c r="K4" s="10">
+      <c r="K4" s="7">
         <f>D5/2</f>
         <v>3175</v>
       </c>
-      <c r="L4" s="10">
+      <c r="L4" s="7">
         <f>D5/2</f>
         <v>3175</v>
       </c>
-      <c r="M4" s="10"/>
-      <c r="N4" s="10"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
     </row>
     <row r="5" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B5" s="14"/>
-      <c r="C5" s="11" t="s">
+      <c r="B5" s="22"/>
+      <c r="C5" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="7">
         <f>3175*2</f>
         <v>6350</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="7">
         <f>SUM(D5)</f>
         <v>6350</v>
       </c>
@@ -1029,50 +1029,50 @@
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
-      <c r="K5" s="10"/>
-      <c r="L5" s="10"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="10"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
     </row>
     <row r="6" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B6" s="14"/>
+      <c r="B6" s="22"/>
       <c r="C6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
-      <c r="K6" s="10">
+      <c r="K6" s="7">
         <f>D7/4</f>
         <v>1161</v>
       </c>
-      <c r="L6" s="10">
+      <c r="L6" s="7">
         <f>D7/4</f>
         <v>1161</v>
       </c>
-      <c r="M6" s="10">
+      <c r="M6" s="7">
         <f>D7/4</f>
         <v>1161</v>
       </c>
-      <c r="N6" s="10">
+      <c r="N6" s="7">
         <f>D7/4</f>
         <v>1161</v>
       </c>
     </row>
     <row r="7" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B7" s="14"/>
-      <c r="C7" s="11" t="s">
+      <c r="B7" s="22"/>
+      <c r="C7" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="7">
         <f>1161*4</f>
         <v>4644</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="7">
         <f>SUM(D7)</f>
         <v>4644</v>
       </c>
@@ -1081,40 +1081,40 @@
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
-      <c r="K7" s="10"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
     </row>
     <row r="8" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B8" s="14"/>
+      <c r="B8" s="22"/>
       <c r="C8" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
-      <c r="K8" s="10">
+      <c r="K8" s="7">
         <f>D9/4</f>
         <v>1158</v>
       </c>
-      <c r="L8" s="10">
+      <c r="L8" s="7">
         <f>D9/4</f>
         <v>1158</v>
       </c>
-      <c r="M8" s="10">
+      <c r="M8" s="7">
         <f>D9/4</f>
         <v>1158</v>
       </c>
-      <c r="N8" s="10">
+      <c r="N8" s="7">
         <f>D9/4</f>
         <v>1158</v>
       </c>
-      <c r="S8" s="25" t="s">
+      <c r="S8" s="14" t="s">
         <v>76</v>
       </c>
       <c r="T8" s="2" t="s">
@@ -1131,15 +1131,15 @@
       </c>
     </row>
     <row r="9" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B9" s="14"/>
-      <c r="C9" s="11" t="s">
+      <c r="B9" s="22"/>
+      <c r="C9" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="7">
         <f>1158*4</f>
         <v>4632</v>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="7">
         <f>SUM(D9)</f>
         <v>4632</v>
       </c>
@@ -1148,11 +1148,11 @@
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10"/>
-      <c r="S9" s="26"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="S9" s="15"/>
       <c r="T9" s="3">
         <f>SUM(K2:K96)</f>
         <v>78934.909999999974</v>
@@ -1165,57 +1165,57 @@
       <c r="W9" s="4"/>
     </row>
     <row r="10" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B10" s="14"/>
+      <c r="B10" s="22"/>
       <c r="C10" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
-      <c r="K10" s="10">
+      <c r="K10" s="7">
         <f>D11/4</f>
         <v>256</v>
       </c>
-      <c r="L10" s="10">
+      <c r="L10" s="7">
         <f>D11/4</f>
         <v>256</v>
       </c>
-      <c r="M10" s="10">
+      <c r="M10" s="7">
         <f>D11/4</f>
         <v>256</v>
       </c>
-      <c r="N10" s="10">
+      <c r="N10" s="7">
         <f>D11/4</f>
         <v>256</v>
       </c>
-      <c r="S10" s="6"/>
-      <c r="T10" s="7"/>
-      <c r="U10" s="7"/>
-      <c r="V10" s="7"/>
-      <c r="W10" s="8"/>
+      <c r="S10" s="16"/>
+      <c r="T10" s="17"/>
+      <c r="U10" s="17"/>
+      <c r="V10" s="17"/>
+      <c r="W10" s="18"/>
     </row>
     <row r="11" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B11" s="14"/>
+      <c r="B11" s="22"/>
       <c r="C11" s="4"/>
-      <c r="D11" s="10">
+      <c r="D11" s="7">
         <f>256*4</f>
         <v>1024</v>
       </c>
-      <c r="E11" s="10"/>
+      <c r="E11" s="7"/>
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="10"/>
-      <c r="N11" s="10"/>
-      <c r="S11" s="13" t="s">
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="S11" s="10" t="s">
         <v>80</v>
       </c>
       <c r="T11" s="2" t="s">
@@ -1232,27 +1232,27 @@
       </c>
     </row>
     <row r="12" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B12" s="14"/>
+      <c r="B12" s="22"/>
       <c r="C12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
       <c r="F12" s="4"/>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
-      <c r="K12" s="10">
+      <c r="K12" s="7">
         <f>D13/2</f>
         <v>340</v>
       </c>
-      <c r="L12" s="10">
+      <c r="L12" s="7">
         <f>D13/2</f>
         <v>340</v>
       </c>
-      <c r="M12" s="10"/>
-      <c r="N12" s="10"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="7"/>
       <c r="S12" s="5">
         <f>SUM(D13,D17,D18,D20,D22,D23,D25,D27,D28,D30,D32,D33,D35,D36,D37,D39,D41,D43,D44,D45,D49,D47,D50,D51,D52,D54,D56,D57,D59,D61,D63,D64,D66,D70,D71,D73,D74,D76,D78,D80,D81,D82,D85,D87,D89,D90)</f>
         <v>58593.979999999996</v>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="U12" s="3">
         <f>SUM(L12,L16,L21,L26,L29,L31,L34,L38,L42,L46,L49,L55,L60,L62,L69,L72,L75,L79,L80,L84,L88,L86)</f>
-        <v>22147.735000000004</v>
+        <v>22147.735000000001</v>
       </c>
       <c r="V12" s="3">
         <f>SUM(M49)</f>
@@ -1275,54 +1275,54 @@
       </c>
     </row>
     <row r="13" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B13" s="14"/>
-      <c r="C13" s="11" t="s">
+      <c r="B13" s="22"/>
+      <c r="C13" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="7">
         <v>680</v>
       </c>
-      <c r="E13" s="10"/>
+      <c r="E13" s="7"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
       <c r="J13" s="4"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="10"/>
-      <c r="N13" s="10"/>
-      <c r="S13" s="6"/>
-      <c r="T13" s="7"/>
-      <c r="U13" s="7"/>
-      <c r="V13" s="7"/>
-      <c r="W13" s="8"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
+      <c r="S13" s="16"/>
+      <c r="T13" s="17"/>
+      <c r="U13" s="17"/>
+      <c r="V13" s="17"/>
+      <c r="W13" s="18"/>
     </row>
     <row r="14" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B14" s="15">
+      <c r="B14" s="23">
         <v>42856</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
       <c r="J14" s="4"/>
-      <c r="K14" s="10">
+      <c r="K14" s="7">
         <f>D15/2</f>
         <v>4229.875</v>
       </c>
-      <c r="L14" s="10">
+      <c r="L14" s="7">
         <f>D15/2</f>
         <v>4229.875</v>
       </c>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10"/>
-      <c r="S14" s="13" t="s">
+      <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
+      <c r="S14" s="10" t="s">
         <v>81</v>
       </c>
       <c r="T14" s="2" t="s">
@@ -1339,24 +1339,24 @@
       </c>
     </row>
     <row r="15" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B15" s="15"/>
-      <c r="C15" s="11" t="s">
+      <c r="B15" s="23"/>
+      <c r="C15" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="7">
         <v>8459.75</v>
       </c>
-      <c r="E15" s="10"/>
+      <c r="E15" s="7"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10"/>
-      <c r="S15" s="9">
+      <c r="K15" s="7"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
+      <c r="N15" s="7"/>
+      <c r="S15" s="6">
         <f>SUM(D15,D68)</f>
         <v>20888.059999999998</v>
       </c>
@@ -1375,158 +1375,158 @@
       <c r="W15" s="4"/>
     </row>
     <row r="16" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B16" s="15"/>
+      <c r="B16" s="23"/>
       <c r="C16" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
       <c r="J16" s="4"/>
-      <c r="K16" s="10">
+      <c r="K16" s="7">
         <f>D18</f>
         <v>509.12</v>
       </c>
-      <c r="L16" s="10">
+      <c r="L16" s="7">
         <f>D17</f>
         <v>423.35</v>
       </c>
-      <c r="M16" s="10"/>
-      <c r="N16" s="10"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="7"/>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B17" s="15"/>
-      <c r="C17" s="11" t="s">
+      <c r="B17" s="23"/>
+      <c r="C17" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D17" s="10">
+      <c r="D17" s="7">
         <v>423.35</v>
       </c>
-      <c r="E17" s="10"/>
+      <c r="E17" s="7"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="10"/>
-      <c r="N17" s="10"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="7"/>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B18" s="15"/>
-      <c r="C18" s="11" t="s">
+      <c r="B18" s="23"/>
+      <c r="C18" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="7">
         <v>509.12</v>
       </c>
-      <c r="E18" s="10"/>
+      <c r="E18" s="7"/>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="10"/>
-      <c r="N18" s="10"/>
+      <c r="K18" s="7"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B19" s="15"/>
+      <c r="B19" s="23"/>
       <c r="C19" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
       <c r="J19" s="4"/>
-      <c r="K19" s="10">
+      <c r="K19" s="7">
         <f>D20</f>
         <v>3330.65</v>
       </c>
-      <c r="L19" s="10"/>
-      <c r="M19" s="10"/>
-      <c r="N19" s="10"/>
+      <c r="L19" s="7"/>
+      <c r="M19" s="7"/>
+      <c r="N19" s="7"/>
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B20" s="15"/>
-      <c r="C20" s="11" t="s">
+      <c r="B20" s="23"/>
+      <c r="C20" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="7">
         <v>3330.65</v>
       </c>
-      <c r="E20" s="10"/>
+      <c r="E20" s="7"/>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
-      <c r="M20" s="10"/>
-      <c r="N20" s="10"/>
+      <c r="K20" s="7"/>
+      <c r="L20" s="7"/>
+      <c r="M20" s="7"/>
+      <c r="N20" s="7"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B21" s="15"/>
+      <c r="B21" s="23"/>
       <c r="C21" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
-      <c r="K21" s="10">
+      <c r="K21" s="7">
         <f>D22</f>
         <v>229.48</v>
       </c>
-      <c r="L21" s="10">
+      <c r="L21" s="7">
         <f>D23</f>
         <v>190.8</v>
       </c>
-      <c r="M21" s="10"/>
-      <c r="N21" s="10"/>
+      <c r="M21" s="7"/>
+      <c r="N21" s="7"/>
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B22" s="15"/>
-      <c r="C22" s="11" t="s">
+      <c r="B22" s="23"/>
+      <c r="C22" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D22" s="10">
+      <c r="D22" s="7">
         <f>220.48+9</f>
         <v>229.48</v>
       </c>
-      <c r="E22" s="10"/>
+      <c r="E22" s="7"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
-      <c r="K22" s="10"/>
-      <c r="L22" s="10"/>
-      <c r="M22" s="10"/>
-      <c r="N22" s="10"/>
+      <c r="K22" s="7"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="7"/>
+      <c r="N22" s="7"/>
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B23" s="15"/>
-      <c r="C23" s="11" t="s">
+      <c r="B23" s="23"/>
+      <c r="C23" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D23" s="10">
+      <c r="D23" s="7">
         <f>181.8+9</f>
         <v>190.8</v>
       </c>
-      <c r="E23" s="10">
+      <c r="E23" s="7">
         <f>SUM(D22,D23)</f>
         <v>420.28</v>
       </c>
@@ -1535,206 +1535,206 @@
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
       <c r="J23" s="4"/>
-      <c r="K23" s="10"/>
-      <c r="L23" s="10"/>
-      <c r="M23" s="10"/>
-      <c r="N23" s="10"/>
+      <c r="K23" s="7"/>
+      <c r="L23" s="7"/>
+      <c r="M23" s="7"/>
+      <c r="N23" s="7"/>
     </row>
     <row r="24" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B24" s="15"/>
+      <c r="B24" s="23"/>
       <c r="C24" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
       <c r="J24" s="4"/>
-      <c r="K24" s="10">
+      <c r="K24" s="7">
         <f>D25</f>
         <v>1331.86</v>
       </c>
-      <c r="L24" s="10"/>
-      <c r="M24" s="10"/>
-      <c r="N24" s="10"/>
+      <c r="L24" s="7"/>
+      <c r="M24" s="7"/>
+      <c r="N24" s="7"/>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B25" s="15"/>
-      <c r="C25" s="11" t="s">
+      <c r="B25" s="23"/>
+      <c r="C25" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D25" s="10">
+      <c r="D25" s="7">
         <v>1331.86</v>
       </c>
-      <c r="E25" s="10"/>
+      <c r="E25" s="7"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
       <c r="J25" s="4"/>
-      <c r="K25" s="10"/>
-      <c r="L25" s="10"/>
-      <c r="M25" s="10"/>
-      <c r="N25" s="10"/>
+      <c r="K25" s="7"/>
+      <c r="L25" s="7"/>
+      <c r="M25" s="7"/>
+      <c r="N25" s="7"/>
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B26" s="15"/>
+      <c r="B26" s="23"/>
       <c r="C26" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
-      <c r="K26" s="10">
+      <c r="K26" s="7">
         <f>D27</f>
         <v>585.75</v>
       </c>
-      <c r="L26" s="10">
+      <c r="L26" s="7">
         <f>D28</f>
         <v>414.87</v>
       </c>
-      <c r="M26" s="10"/>
-      <c r="N26" s="10"/>
+      <c r="M26" s="7"/>
+      <c r="N26" s="7"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B27" s="15"/>
-      <c r="C27" s="11" t="s">
+      <c r="B27" s="23"/>
+      <c r="C27" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D27" s="10">
+      <c r="D27" s="7">
         <v>585.75</v>
       </c>
-      <c r="E27" s="10"/>
+      <c r="E27" s="7"/>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
-      <c r="K27" s="10"/>
-      <c r="L27" s="10"/>
-      <c r="M27" s="10"/>
-      <c r="N27" s="10"/>
+      <c r="K27" s="7"/>
+      <c r="L27" s="7"/>
+      <c r="M27" s="7"/>
+      <c r="N27" s="7"/>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B28" s="15"/>
-      <c r="C28" s="11" t="s">
+      <c r="B28" s="23"/>
+      <c r="C28" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D28" s="10">
+      <c r="D28" s="7">
         <v>414.87</v>
       </c>
-      <c r="E28" s="10"/>
+      <c r="E28" s="7"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
-      <c r="K28" s="10"/>
-      <c r="L28" s="10"/>
-      <c r="M28" s="10"/>
-      <c r="N28" s="10"/>
+      <c r="K28" s="7"/>
+      <c r="L28" s="7"/>
+      <c r="M28" s="7"/>
+      <c r="N28" s="7"/>
     </row>
     <row r="29" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B29" s="15"/>
+      <c r="B29" s="23"/>
       <c r="C29" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
       <c r="I29" s="4"/>
       <c r="J29" s="4"/>
-      <c r="K29" s="10">
+      <c r="K29" s="7">
         <f>D30/2</f>
         <v>275.05</v>
       </c>
-      <c r="L29" s="10">
+      <c r="L29" s="7">
         <f>D30/2</f>
         <v>275.05</v>
       </c>
-      <c r="M29" s="10"/>
-      <c r="N29" s="10"/>
+      <c r="M29" s="7"/>
+      <c r="N29" s="7"/>
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B30" s="15"/>
-      <c r="C30" s="11" t="s">
+      <c r="B30" s="23"/>
+      <c r="C30" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D30" s="7">
         <v>550.1</v>
       </c>
-      <c r="E30" s="10"/>
+      <c r="E30" s="7"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
       <c r="J30" s="4"/>
-      <c r="K30" s="10"/>
-      <c r="L30" s="10"/>
-      <c r="M30" s="10"/>
-      <c r="N30" s="10"/>
+      <c r="K30" s="7"/>
+      <c r="L30" s="7"/>
+      <c r="M30" s="7"/>
+      <c r="N30" s="7"/>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B31" s="15"/>
+      <c r="B31" s="23"/>
       <c r="C31" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
       <c r="J31" s="4"/>
-      <c r="K31" s="10">
+      <c r="K31" s="7">
         <f>D32</f>
         <v>6075.6</v>
       </c>
-      <c r="L31" s="10">
+      <c r="L31" s="7">
         <f>D33</f>
         <v>6462.6</v>
       </c>
-      <c r="M31" s="10"/>
-      <c r="N31" s="10"/>
+      <c r="M31" s="7"/>
+      <c r="N31" s="7"/>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B32" s="15"/>
-      <c r="C32" s="11" t="s">
+      <c r="B32" s="23"/>
+      <c r="C32" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D32" s="10">
+      <c r="D32" s="7">
         <f>5801+274.6</f>
         <v>6075.6</v>
       </c>
-      <c r="E32" s="10"/>
+      <c r="E32" s="7"/>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
       <c r="J32" s="4"/>
-      <c r="K32" s="10"/>
-      <c r="L32" s="10"/>
-      <c r="M32" s="10"/>
-      <c r="N32" s="10"/>
+      <c r="K32" s="7"/>
+      <c r="L32" s="7"/>
+      <c r="M32" s="7"/>
+      <c r="N32" s="7"/>
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B33" s="15"/>
-      <c r="C33" s="11" t="s">
+      <c r="B33" s="23"/>
+      <c r="C33" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D33" s="10">
+      <c r="D33" s="7">
         <f>6188+274.6</f>
         <v>6462.6</v>
       </c>
-      <c r="E33" s="10">
+      <c r="E33" s="7">
         <f>SUM(D32:D33)</f>
         <v>12538.2</v>
       </c>
@@ -1743,87 +1743,87 @@
       <c r="H33" s="4"/>
       <c r="I33" s="4"/>
       <c r="J33" s="4"/>
-      <c r="K33" s="10"/>
-      <c r="L33" s="10"/>
-      <c r="M33" s="10"/>
-      <c r="N33" s="10"/>
+      <c r="K33" s="7"/>
+      <c r="L33" s="7"/>
+      <c r="M33" s="7"/>
+      <c r="N33" s="7"/>
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B34" s="15"/>
+      <c r="B34" s="23"/>
       <c r="C34" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
       <c r="I34" s="4"/>
       <c r="J34" s="4"/>
-      <c r="K34" s="10">
+      <c r="K34" s="7">
         <f>D36</f>
         <v>1003.4300000000001</v>
       </c>
-      <c r="L34" s="10">
+      <c r="L34" s="7">
         <f>D37</f>
         <v>1364.9699999999998</v>
       </c>
-      <c r="M34" s="10"/>
-      <c r="N34" s="10">
+      <c r="M34" s="7"/>
+      <c r="N34" s="7">
         <f>D35</f>
         <v>386.09000000000003</v>
       </c>
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B35" s="15"/>
-      <c r="C35" s="11" t="s">
+      <c r="B35" s="23"/>
+      <c r="C35" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D35" s="10">
+      <c r="D35" s="7">
         <f>345.8+40.29</f>
         <v>386.09000000000003</v>
       </c>
-      <c r="E35" s="10"/>
+      <c r="E35" s="7"/>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
       <c r="I35" s="4"/>
       <c r="J35" s="4"/>
-      <c r="K35" s="10"/>
-      <c r="L35" s="10"/>
-      <c r="M35" s="10"/>
-      <c r="N35" s="10"/>
+      <c r="K35" s="7"/>
+      <c r="L35" s="7"/>
+      <c r="M35" s="7"/>
+      <c r="N35" s="7"/>
     </row>
     <row r="36" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B36" s="15"/>
-      <c r="C36" s="11" t="s">
+      <c r="B36" s="23"/>
+      <c r="C36" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D36" s="10">
+      <c r="D36" s="7">
         <f>345.8+308.67*2+40.29</f>
         <v>1003.4300000000001</v>
       </c>
-      <c r="E36" s="10"/>
+      <c r="E36" s="7"/>
       <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
-      <c r="K36" s="10"/>
-      <c r="L36" s="10"/>
-      <c r="M36" s="10"/>
-      <c r="N36" s="10"/>
+      <c r="K36" s="7"/>
+      <c r="L36" s="7"/>
+      <c r="M36" s="7"/>
+      <c r="N36" s="7"/>
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B37" s="15"/>
-      <c r="C37" s="11" t="s">
+      <c r="B37" s="23"/>
+      <c r="C37" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D37" s="10">
+      <c r="D37" s="7">
         <f>308.67+192.63+483+340.38+40.29</f>
         <v>1364.9699999999998</v>
       </c>
-      <c r="E37" s="10">
+      <c r="E37" s="7">
         <v>2754.49</v>
       </c>
       <c r="F37" s="4"/>
@@ -1831,316 +1831,316 @@
       <c r="H37" s="4"/>
       <c r="I37" s="4"/>
       <c r="J37" s="4"/>
-      <c r="K37" s="10"/>
-      <c r="L37" s="10"/>
-      <c r="M37" s="10"/>
-      <c r="N37" s="10"/>
+      <c r="K37" s="7"/>
+      <c r="L37" s="7"/>
+      <c r="M37" s="7"/>
+      <c r="N37" s="7"/>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B38" s="16">
+      <c r="B38" s="24">
         <v>43221</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D38" s="10"/>
-      <c r="E38" s="10"/>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
       <c r="J38" s="4"/>
-      <c r="K38" s="10">
+      <c r="K38" s="7">
         <f>D39/2</f>
         <v>135.36500000000001</v>
       </c>
-      <c r="L38" s="10">
+      <c r="L38" s="7">
         <f>D39/2</f>
         <v>135.36500000000001</v>
       </c>
-      <c r="M38" s="10"/>
-      <c r="N38" s="10"/>
+      <c r="M38" s="7"/>
+      <c r="N38" s="7"/>
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B39" s="16"/>
+      <c r="B39" s="24"/>
       <c r="C39" s="4"/>
-      <c r="D39" s="10">
+      <c r="D39" s="7">
         <v>270.73</v>
       </c>
-      <c r="E39" s="10"/>
+      <c r="E39" s="7"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
-      <c r="K39" s="10"/>
-      <c r="L39" s="10"/>
-      <c r="M39" s="10"/>
-      <c r="N39" s="10"/>
+      <c r="K39" s="7"/>
+      <c r="L39" s="7"/>
+      <c r="M39" s="7"/>
+      <c r="N39" s="7"/>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B40" s="17">
+      <c r="B40" s="25">
         <v>43586</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D40" s="10"/>
-      <c r="E40" s="10"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
-      <c r="K40" s="10">
+      <c r="K40" s="7">
         <f>D41</f>
         <v>1129.3499999999999</v>
       </c>
-      <c r="L40" s="10"/>
-      <c r="M40" s="10"/>
-      <c r="N40" s="10"/>
+      <c r="L40" s="7"/>
+      <c r="M40" s="7"/>
+      <c r="N40" s="7"/>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B41" s="17"/>
+      <c r="B41" s="25"/>
       <c r="C41" s="4"/>
-      <c r="D41" s="10">
+      <c r="D41" s="7">
         <v>1129.3499999999999</v>
       </c>
-      <c r="E41" s="10"/>
+      <c r="E41" s="7"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
       <c r="I41" s="4"/>
       <c r="J41" s="4"/>
-      <c r="K41" s="10"/>
-      <c r="L41" s="10"/>
-      <c r="M41" s="10"/>
-      <c r="N41" s="10"/>
+      <c r="K41" s="7"/>
+      <c r="L41" s="7"/>
+      <c r="M41" s="7"/>
+      <c r="N41" s="7"/>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B42" s="17"/>
+      <c r="B42" s="25"/>
       <c r="C42" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D42" s="10"/>
-      <c r="E42" s="10"/>
+      <c r="D42" s="7"/>
+      <c r="E42" s="7"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
-      <c r="K42" s="10">
+      <c r="K42" s="7">
         <f>D44</f>
         <v>636.72</v>
       </c>
-      <c r="L42" s="10">
+      <c r="L42" s="7">
         <f>D43</f>
         <v>980.92</v>
       </c>
-      <c r="M42" s="10"/>
-      <c r="N42" s="10">
+      <c r="M42" s="7"/>
+      <c r="N42" s="7">
         <f>D45</f>
         <v>78</v>
       </c>
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B43" s="17"/>
-      <c r="C43" s="11" t="s">
+      <c r="B43" s="25"/>
+      <c r="C43" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="D43" s="10">
+      <c r="D43" s="7">
         <v>980.92</v>
       </c>
-      <c r="E43" s="10"/>
+      <c r="E43" s="7"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
       <c r="J43" s="4"/>
-      <c r="K43" s="10"/>
-      <c r="L43" s="10"/>
-      <c r="M43" s="10"/>
-      <c r="N43" s="10"/>
+      <c r="K43" s="7"/>
+      <c r="L43" s="7"/>
+      <c r="M43" s="7"/>
+      <c r="N43" s="7"/>
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B44" s="17"/>
-      <c r="C44" s="11" t="s">
+      <c r="B44" s="25"/>
+      <c r="C44" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D44" s="10">
+      <c r="D44" s="7">
         <v>636.72</v>
       </c>
-      <c r="E44" s="10"/>
+      <c r="E44" s="7"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
       <c r="I44" s="4"/>
       <c r="J44" s="4"/>
-      <c r="K44" s="10"/>
-      <c r="L44" s="10"/>
-      <c r="M44" s="10"/>
-      <c r="N44" s="10"/>
+      <c r="K44" s="7"/>
+      <c r="L44" s="7"/>
+      <c r="M44" s="7"/>
+      <c r="N44" s="7"/>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B45" s="17"/>
-      <c r="C45" s="11" t="s">
+      <c r="B45" s="25"/>
+      <c r="C45" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D45" s="10">
+      <c r="D45" s="7">
         <v>78</v>
       </c>
-      <c r="E45" s="10"/>
+      <c r="E45" s="7"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
       <c r="I45" s="4"/>
       <c r="J45" s="4"/>
-      <c r="K45" s="10"/>
-      <c r="L45" s="10"/>
-      <c r="M45" s="10"/>
-      <c r="N45" s="10"/>
+      <c r="K45" s="7"/>
+      <c r="L45" s="7"/>
+      <c r="M45" s="7"/>
+      <c r="N45" s="7"/>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B46" s="17"/>
+      <c r="B46" s="25"/>
       <c r="C46" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D46" s="10"/>
-      <c r="E46" s="10"/>
+      <c r="D46" s="7"/>
+      <c r="E46" s="7"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
       <c r="I46" s="4"/>
       <c r="J46" s="4"/>
-      <c r="K46" s="10">
+      <c r="K46" s="7">
         <f>D47/2</f>
         <v>471.02</v>
       </c>
-      <c r="L46" s="10">
+      <c r="L46" s="7">
         <f>D47/2</f>
         <v>471.02</v>
       </c>
-      <c r="M46" s="10"/>
-      <c r="N46" s="10"/>
+      <c r="M46" s="7"/>
+      <c r="N46" s="7"/>
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B47" s="17"/>
-      <c r="C47" s="11" t="s">
+      <c r="B47" s="25"/>
+      <c r="C47" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="D47" s="10">
+      <c r="D47" s="7">
         <v>942.04</v>
       </c>
-      <c r="E47" s="10"/>
+      <c r="E47" s="7"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
       <c r="I47" s="4"/>
       <c r="J47" s="4"/>
-      <c r="K47" s="10"/>
-      <c r="L47" s="10"/>
-      <c r="M47" s="10"/>
-      <c r="N47" s="10"/>
+      <c r="K47" s="7"/>
+      <c r="L47" s="7"/>
+      <c r="M47" s="7"/>
+      <c r="N47" s="7"/>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B48" s="17"/>
+      <c r="B48" s="25"/>
       <c r="C48" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D48" s="10"/>
-      <c r="E48" s="10"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
       <c r="I48" s="4"/>
       <c r="J48" s="4"/>
-      <c r="K48" s="10"/>
-      <c r="L48" s="10"/>
-      <c r="M48" s="10"/>
-      <c r="N48" s="10"/>
+      <c r="K48" s="7"/>
+      <c r="L48" s="7"/>
+      <c r="M48" s="7"/>
+      <c r="N48" s="7"/>
     </row>
     <row r="49" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B49" s="17"/>
-      <c r="C49" s="11" t="s">
+      <c r="B49" s="25"/>
+      <c r="C49" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="D49" s="10">
+      <c r="D49" s="7">
         <f>243.64+11.055</f>
         <v>254.69499999999999</v>
       </c>
-      <c r="E49" s="10"/>
+      <c r="E49" s="7"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="4"/>
       <c r="I49" s="4"/>
       <c r="J49" s="4"/>
-      <c r="K49" s="10">
+      <c r="K49" s="7">
         <f>D50</f>
         <v>262.42500000000001</v>
       </c>
-      <c r="L49" s="10">
+      <c r="L49" s="7">
         <f>D49</f>
         <v>254.69499999999999</v>
       </c>
-      <c r="M49" s="10">
+      <c r="M49" s="7">
         <f>D52</f>
         <v>262.42500000000001</v>
       </c>
-      <c r="N49" s="10">
+      <c r="N49" s="7">
         <f>D51</f>
         <v>250.82500000000002</v>
       </c>
     </row>
     <row r="50" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B50" s="17"/>
-      <c r="C50" s="11" t="s">
+      <c r="B50" s="25"/>
+      <c r="C50" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D50" s="10">
+      <c r="D50" s="7">
         <f>251.37+11.055</f>
         <v>262.42500000000001</v>
       </c>
-      <c r="E50" s="10"/>
+      <c r="E50" s="7"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
       <c r="I50" s="4"/>
       <c r="J50" s="4"/>
-      <c r="K50" s="10"/>
-      <c r="L50" s="10"/>
-      <c r="M50" s="10"/>
-      <c r="N50" s="10"/>
+      <c r="K50" s="7"/>
+      <c r="L50" s="7"/>
+      <c r="M50" s="7"/>
+      <c r="N50" s="7"/>
     </row>
     <row r="51" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B51" s="17"/>
-      <c r="C51" s="11" t="s">
+      <c r="B51" s="25"/>
+      <c r="C51" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D51" s="10">
+      <c r="D51" s="7">
         <f>239.77+11.055</f>
         <v>250.82500000000002</v>
       </c>
-      <c r="E51" s="10"/>
+      <c r="E51" s="7"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
       <c r="I51" s="4"/>
       <c r="J51" s="4"/>
-      <c r="K51" s="10"/>
-      <c r="L51" s="10"/>
-      <c r="M51" s="10"/>
-      <c r="N51" s="10"/>
+      <c r="K51" s="7"/>
+      <c r="L51" s="7"/>
+      <c r="M51" s="7"/>
+      <c r="N51" s="7"/>
     </row>
     <row r="52" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B52" s="17"/>
-      <c r="C52" s="11" t="s">
+      <c r="B52" s="25"/>
+      <c r="C52" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="D52" s="10">
+      <c r="D52" s="7">
         <f>251.37+11.055</f>
         <v>262.42500000000001</v>
       </c>
-      <c r="E52" s="10">
+      <c r="E52" s="7">
         <f>SUM(D49:D52)</f>
         <v>1030.3700000000001</v>
       </c>
@@ -2149,101 +2149,101 @@
       <c r="H52" s="4"/>
       <c r="I52" s="4"/>
       <c r="J52" s="4"/>
-      <c r="K52" s="10"/>
-      <c r="L52" s="10"/>
-      <c r="M52" s="10"/>
-      <c r="N52" s="10"/>
+      <c r="K52" s="7"/>
+      <c r="L52" s="7"/>
+      <c r="M52" s="7"/>
+      <c r="N52" s="7"/>
     </row>
     <row r="53" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B53" s="17"/>
+      <c r="B53" s="25"/>
       <c r="C53" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D53" s="10"/>
-      <c r="E53" s="10"/>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
       <c r="I53" s="4"/>
       <c r="J53" s="4"/>
-      <c r="K53" s="10">
+      <c r="K53" s="7">
         <f>D54</f>
         <v>197.99</v>
       </c>
-      <c r="L53" s="10"/>
-      <c r="M53" s="10"/>
-      <c r="N53" s="10"/>
+      <c r="L53" s="7"/>
+      <c r="M53" s="7"/>
+      <c r="N53" s="7"/>
     </row>
     <row r="54" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B54" s="17"/>
-      <c r="C54" s="11" t="s">
+      <c r="B54" s="25"/>
+      <c r="C54" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D54" s="10">
+      <c r="D54" s="7">
         <v>197.99</v>
       </c>
-      <c r="E54" s="10"/>
+      <c r="E54" s="7"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
       <c r="I54" s="4"/>
       <c r="J54" s="4"/>
-      <c r="K54" s="10"/>
-      <c r="L54" s="10"/>
-      <c r="M54" s="10"/>
-      <c r="N54" s="10"/>
+      <c r="K54" s="7"/>
+      <c r="L54" s="7"/>
+      <c r="M54" s="7"/>
+      <c r="N54" s="7"/>
     </row>
     <row r="55" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B55" s="17"/>
-      <c r="C55" s="12" t="s">
+      <c r="B55" s="25"/>
+      <c r="C55" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="D55" s="10"/>
-      <c r="E55" s="10"/>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
       <c r="I55" s="4"/>
       <c r="J55" s="4"/>
-      <c r="K55" s="10">
+      <c r="K55" s="7">
         <f>D56</f>
         <v>6000.1</v>
       </c>
-      <c r="L55" s="10">
+      <c r="L55" s="7">
         <f>D57</f>
         <v>6000.1</v>
       </c>
-      <c r="M55" s="10"/>
-      <c r="N55" s="10"/>
+      <c r="M55" s="7"/>
+      <c r="N55" s="7"/>
     </row>
     <row r="56" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B56" s="17"/>
-      <c r="C56" s="11" t="s">
+      <c r="B56" s="25"/>
+      <c r="C56" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D56" s="10">
+      <c r="D56" s="7">
         <v>6000.1</v>
       </c>
-      <c r="E56" s="10"/>
+      <c r="E56" s="7"/>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
       <c r="I56" s="4"/>
       <c r="J56" s="4"/>
-      <c r="K56" s="10"/>
-      <c r="L56" s="10"/>
-      <c r="M56" s="10"/>
-      <c r="N56" s="10"/>
+      <c r="K56" s="7"/>
+      <c r="L56" s="7"/>
+      <c r="M56" s="7"/>
+      <c r="N56" s="7"/>
     </row>
     <row r="57" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B57" s="17"/>
-      <c r="C57" s="11" t="s">
+      <c r="B57" s="25"/>
+      <c r="C57" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D57" s="10">
+      <c r="D57" s="7">
         <v>6000.1</v>
       </c>
-      <c r="E57" s="10">
+      <c r="E57" s="7">
         <v>12100.19</v>
       </c>
       <c r="F57" s="4"/>
@@ -2251,147 +2251,147 @@
       <c r="H57" s="4"/>
       <c r="I57" s="4"/>
       <c r="J57" s="4"/>
-      <c r="K57" s="10"/>
-      <c r="L57" s="10"/>
-      <c r="M57" s="10"/>
-      <c r="N57" s="10"/>
+      <c r="K57" s="7"/>
+      <c r="L57" s="7"/>
+      <c r="M57" s="7"/>
+      <c r="N57" s="7"/>
     </row>
     <row r="58" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B58" s="18">
+      <c r="B58" s="26">
         <v>43952</v>
       </c>
-      <c r="C58" s="12" t="s">
+      <c r="C58" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D58" s="10"/>
-      <c r="E58" s="10"/>
+      <c r="D58" s="7"/>
+      <c r="E58" s="7"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
       <c r="I58" s="4"/>
       <c r="J58" s="4"/>
-      <c r="K58" s="10">
+      <c r="K58" s="7">
         <f>D59</f>
         <v>726.02</v>
       </c>
-      <c r="L58" s="10"/>
-      <c r="M58" s="10"/>
-      <c r="N58" s="10"/>
+      <c r="L58" s="7"/>
+      <c r="M58" s="7"/>
+      <c r="N58" s="7"/>
     </row>
     <row r="59" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B59" s="18"/>
-      <c r="C59" s="11" t="s">
+      <c r="B59" s="26"/>
+      <c r="C59" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="D59" s="10">
+      <c r="D59" s="7">
         <v>726.02</v>
       </c>
-      <c r="E59" s="10"/>
+      <c r="E59" s="7"/>
       <c r="F59" s="4"/>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
       <c r="I59" s="4"/>
       <c r="J59" s="4"/>
-      <c r="K59" s="10"/>
-      <c r="L59" s="10"/>
-      <c r="M59" s="10"/>
-      <c r="N59" s="10"/>
+      <c r="K59" s="7"/>
+      <c r="L59" s="7"/>
+      <c r="M59" s="7"/>
+      <c r="N59" s="7"/>
     </row>
     <row r="60" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B60" s="18"/>
-      <c r="C60" s="12" t="s">
+      <c r="B60" s="26"/>
+      <c r="C60" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D60" s="10"/>
-      <c r="E60" s="10"/>
+      <c r="D60" s="7"/>
+      <c r="E60" s="7"/>
       <c r="F60" s="4"/>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
       <c r="I60" s="4"/>
       <c r="J60" s="4"/>
-      <c r="K60" s="10">
+      <c r="K60" s="7">
         <f>D61/2</f>
         <v>806.68</v>
       </c>
-      <c r="L60" s="10">
+      <c r="L60" s="7">
         <f>D61/2</f>
         <v>806.68</v>
       </c>
-      <c r="M60" s="10"/>
-      <c r="N60" s="10"/>
+      <c r="M60" s="7"/>
+      <c r="N60" s="7"/>
     </row>
     <row r="61" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B61" s="18"/>
-      <c r="C61" s="11" t="s">
+      <c r="B61" s="26"/>
+      <c r="C61" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="D61" s="10">
+      <c r="D61" s="7">
         <v>1613.36</v>
       </c>
-      <c r="E61" s="10"/>
+      <c r="E61" s="7"/>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
       <c r="H61" s="4"/>
       <c r="I61" s="4"/>
       <c r="J61" s="4"/>
-      <c r="K61" s="10"/>
-      <c r="L61" s="10"/>
-      <c r="M61" s="10"/>
-      <c r="N61" s="10"/>
+      <c r="K61" s="7"/>
+      <c r="L61" s="7"/>
+      <c r="M61" s="7"/>
+      <c r="N61" s="7"/>
     </row>
     <row r="62" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B62" s="18"/>
-      <c r="C62" s="12" t="s">
+      <c r="B62" s="26"/>
+      <c r="C62" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D62" s="10"/>
-      <c r="E62" s="10"/>
+      <c r="D62" s="7"/>
+      <c r="E62" s="7"/>
       <c r="F62" s="4"/>
       <c r="G62" s="4"/>
       <c r="H62" s="4"/>
       <c r="I62" s="4"/>
       <c r="J62" s="4"/>
-      <c r="K62" s="10">
+      <c r="K62" s="7">
         <f>D64</f>
         <v>297.89999999999998</v>
       </c>
-      <c r="L62" s="10">
+      <c r="L62" s="7">
         <f>D63</f>
         <v>274.89999999999998</v>
       </c>
-      <c r="M62" s="10"/>
-      <c r="N62" s="10"/>
+      <c r="M62" s="7"/>
+      <c r="N62" s="7"/>
     </row>
     <row r="63" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B63" s="18"/>
-      <c r="C63" s="11" t="s">
+      <c r="B63" s="26"/>
+      <c r="C63" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D63" s="10">
+      <c r="D63" s="7">
         <f>263+11.9</f>
         <v>274.89999999999998</v>
       </c>
-      <c r="E63" s="10"/>
+      <c r="E63" s="7"/>
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
       <c r="I63" s="4"/>
       <c r="J63" s="4"/>
-      <c r="K63" s="10"/>
-      <c r="L63" s="10"/>
-      <c r="M63" s="10"/>
-      <c r="N63" s="10"/>
+      <c r="K63" s="7"/>
+      <c r="L63" s="7"/>
+      <c r="M63" s="7"/>
+      <c r="N63" s="7"/>
     </row>
     <row r="64" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B64" s="18"/>
-      <c r="C64" s="11" t="s">
+      <c r="B64" s="26"/>
+      <c r="C64" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D64" s="10">
+      <c r="D64" s="7">
         <f>286+11.9</f>
         <v>297.89999999999998</v>
       </c>
-      <c r="E64" s="10">
+      <c r="E64" s="7">
         <v>572.73</v>
       </c>
       <c r="F64" s="4"/>
@@ -2399,152 +2399,152 @@
       <c r="H64" s="4"/>
       <c r="I64" s="4"/>
       <c r="J64" s="4"/>
-      <c r="K64" s="10"/>
-      <c r="L64" s="10"/>
-      <c r="M64" s="10"/>
-      <c r="N64" s="10"/>
+      <c r="K64" s="7"/>
+      <c r="L64" s="7"/>
+      <c r="M64" s="7"/>
+      <c r="N64" s="7"/>
     </row>
     <row r="65" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B65" s="19">
         <v>44317</v>
       </c>
-      <c r="C65" s="12" t="s">
+      <c r="C65" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="D65" s="10"/>
-      <c r="E65" s="10"/>
+      <c r="D65" s="7"/>
+      <c r="E65" s="7"/>
       <c r="F65" s="4"/>
       <c r="G65" s="4"/>
       <c r="H65" s="4"/>
       <c r="I65" s="4"/>
       <c r="J65" s="4"/>
-      <c r="K65" s="10">
+      <c r="K65" s="7">
         <f>D66</f>
         <v>2196.59</v>
       </c>
-      <c r="L65" s="10"/>
-      <c r="M65" s="10"/>
-      <c r="N65" s="10"/>
+      <c r="L65" s="7"/>
+      <c r="M65" s="7"/>
+      <c r="N65" s="7"/>
     </row>
     <row r="66" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B66" s="19"/>
-      <c r="C66" s="11" t="s">
+      <c r="C66" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="D66" s="10">
+      <c r="D66" s="7">
         <v>2196.59</v>
       </c>
-      <c r="E66" s="10"/>
+      <c r="E66" s="7"/>
       <c r="F66" s="4"/>
       <c r="G66" s="4"/>
       <c r="H66" s="4"/>
       <c r="I66" s="4"/>
       <c r="J66" s="4"/>
-      <c r="K66" s="10"/>
-      <c r="L66" s="10"/>
-      <c r="M66" s="10"/>
-      <c r="N66" s="10"/>
+      <c r="K66" s="7"/>
+      <c r="L66" s="7"/>
+      <c r="M66" s="7"/>
+      <c r="N66" s="7"/>
     </row>
     <row r="67" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B67" s="19"/>
-      <c r="C67" s="12" t="s">
+      <c r="C67" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D67" s="10"/>
-      <c r="E67" s="10"/>
+      <c r="D67" s="7"/>
+      <c r="E67" s="7"/>
       <c r="F67" s="4"/>
       <c r="G67" s="4"/>
       <c r="H67" s="4"/>
       <c r="I67" s="4"/>
       <c r="J67" s="4"/>
-      <c r="K67" s="10">
+      <c r="K67" s="7">
         <f>D68/3</f>
         <v>4142.7699999999995</v>
       </c>
-      <c r="L67" s="10">
+      <c r="L67" s="7">
         <f>D68/3</f>
         <v>4142.7699999999995</v>
       </c>
-      <c r="M67" s="10">
+      <c r="M67" s="7">
         <f>D68/3</f>
         <v>4142.7699999999995</v>
       </c>
-      <c r="N67" s="10"/>
+      <c r="N67" s="7"/>
     </row>
     <row r="68" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B68" s="19"/>
-      <c r="C68" s="11" t="s">
+      <c r="C68" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="D68" s="10">
+      <c r="D68" s="7">
         <v>12428.31</v>
       </c>
-      <c r="E68" s="10"/>
+      <c r="E68" s="7"/>
       <c r="F68" s="4"/>
       <c r="G68" s="4"/>
       <c r="H68" s="4"/>
       <c r="I68" s="4"/>
       <c r="J68" s="4"/>
-      <c r="K68" s="10"/>
-      <c r="L68" s="10"/>
-      <c r="M68" s="10"/>
-      <c r="N68" s="10"/>
+      <c r="K68" s="7"/>
+      <c r="L68" s="7"/>
+      <c r="M68" s="7"/>
+      <c r="N68" s="7"/>
     </row>
     <row r="69" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B69" s="20">
         <v>44682</v>
       </c>
-      <c r="C69" s="12" t="s">
+      <c r="C69" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="D69" s="10"/>
-      <c r="E69" s="10"/>
+      <c r="D69" s="7"/>
+      <c r="E69" s="7"/>
       <c r="F69" s="4"/>
       <c r="G69" s="4"/>
       <c r="H69" s="4"/>
       <c r="I69" s="4"/>
       <c r="J69" s="4"/>
-      <c r="K69" s="10">
+      <c r="K69" s="7">
         <f>D71</f>
         <v>268.59000000000003</v>
       </c>
-      <c r="L69" s="10">
+      <c r="L69" s="7">
         <f>D70</f>
         <v>280.95000000000005</v>
       </c>
-      <c r="M69" s="10"/>
-      <c r="N69" s="10"/>
+      <c r="M69" s="7"/>
+      <c r="N69" s="7"/>
     </row>
     <row r="70" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B70" s="20"/>
-      <c r="C70" s="11" t="s">
+      <c r="C70" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D70" s="10">
+      <c r="D70" s="7">
         <f>246.11+34.84</f>
         <v>280.95000000000005</v>
       </c>
-      <c r="E70" s="10"/>
+      <c r="E70" s="7"/>
       <c r="F70" s="4"/>
       <c r="G70" s="4"/>
       <c r="H70" s="4"/>
       <c r="I70" s="4"/>
       <c r="J70" s="4"/>
-      <c r="K70" s="10"/>
-      <c r="L70" s="10"/>
-      <c r="M70" s="10"/>
-      <c r="N70" s="10"/>
+      <c r="K70" s="7"/>
+      <c r="L70" s="7"/>
+      <c r="M70" s="7"/>
+      <c r="N70" s="7"/>
     </row>
     <row r="71" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B71" s="20"/>
-      <c r="C71" s="11" t="s">
+      <c r="C71" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D71" s="10">
+      <c r="D71" s="7">
         <f>233.75+34.84</f>
         <v>268.59000000000003</v>
       </c>
-      <c r="E71" s="10">
+      <c r="E71" s="7">
         <v>549.54</v>
       </c>
       <c r="F71" s="4"/>
@@ -2552,62 +2552,62 @@
       <c r="H71" s="4"/>
       <c r="I71" s="4"/>
       <c r="J71" s="4"/>
-      <c r="K71" s="10"/>
-      <c r="L71" s="10"/>
-      <c r="M71" s="10"/>
-      <c r="N71" s="10"/>
+      <c r="K71" s="7"/>
+      <c r="L71" s="7"/>
+      <c r="M71" s="7"/>
+      <c r="N71" s="7"/>
     </row>
     <row r="72" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B72" s="20"/>
-      <c r="C72" s="12" t="s">
+      <c r="C72" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D72" s="10"/>
-      <c r="E72" s="10"/>
+      <c r="D72" s="7"/>
+      <c r="E72" s="7"/>
       <c r="F72" s="4"/>
       <c r="G72" s="4"/>
       <c r="H72" s="4"/>
       <c r="I72" s="4"/>
       <c r="J72" s="4"/>
-      <c r="K72" s="10">
+      <c r="K72" s="7">
         <f>D73</f>
         <v>708.05</v>
       </c>
-      <c r="L72" s="10">
+      <c r="L72" s="7">
         <f>D74</f>
         <v>531.04</v>
       </c>
-      <c r="M72" s="10"/>
-      <c r="N72" s="10"/>
+      <c r="M72" s="7"/>
+      <c r="N72" s="7"/>
     </row>
     <row r="73" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B73" s="20"/>
-      <c r="C73" s="11" t="s">
+      <c r="C73" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="D73" s="10">
+      <c r="D73" s="7">
         <v>708.05</v>
       </c>
-      <c r="E73" s="10"/>
+      <c r="E73" s="7"/>
       <c r="F73" s="4"/>
       <c r="G73" s="4"/>
       <c r="H73" s="4"/>
       <c r="I73" s="4"/>
       <c r="J73" s="4"/>
-      <c r="K73" s="10"/>
-      <c r="L73" s="10"/>
-      <c r="M73" s="10"/>
-      <c r="N73" s="10"/>
+      <c r="K73" s="7"/>
+      <c r="L73" s="7"/>
+      <c r="M73" s="7"/>
+      <c r="N73" s="7"/>
     </row>
     <row r="74" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B74" s="20"/>
-      <c r="C74" s="11" t="s">
+      <c r="C74" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D74" s="10">
+      <c r="D74" s="7">
         <v>531.04</v>
       </c>
-      <c r="E74" s="10">
+      <c r="E74" s="7">
         <f>SUM(D73:D74)</f>
         <v>1239.0899999999999</v>
       </c>
@@ -2616,43 +2616,43 @@
       <c r="H74" s="4"/>
       <c r="I74" s="4"/>
       <c r="J74" s="4"/>
-      <c r="K74" s="10"/>
-      <c r="L74" s="10"/>
-      <c r="M74" s="10"/>
-      <c r="N74" s="10"/>
+      <c r="K74" s="7"/>
+      <c r="L74" s="7"/>
+      <c r="M74" s="7"/>
+      <c r="N74" s="7"/>
     </row>
     <row r="75" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B75" s="20"/>
-      <c r="C75" s="11" t="s">
+      <c r="C75" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="D75" s="10"/>
-      <c r="E75" s="10"/>
+      <c r="D75" s="7"/>
+      <c r="E75" s="7"/>
       <c r="F75" s="4"/>
       <c r="G75" s="4"/>
       <c r="H75" s="4"/>
       <c r="I75" s="4"/>
       <c r="J75" s="4"/>
-      <c r="K75" s="10">
+      <c r="K75" s="7">
         <f>D76/2</f>
         <v>80.265000000000001</v>
       </c>
-      <c r="L75" s="10">
+      <c r="L75" s="7">
         <f>D76/2</f>
         <v>80.265000000000001</v>
       </c>
-      <c r="M75" s="10"/>
-      <c r="N75" s="10"/>
+      <c r="M75" s="7"/>
+      <c r="N75" s="7"/>
     </row>
     <row r="76" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B76" s="20"/>
-      <c r="C76" s="11" t="s">
+      <c r="C76" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="D76" s="10">
+      <c r="D76" s="7">
         <v>160.53</v>
       </c>
-      <c r="E76" s="10">
+      <c r="E76" s="7">
         <f>D76</f>
         <v>160.53</v>
       </c>
@@ -2661,40 +2661,40 @@
       <c r="H76" s="4"/>
       <c r="I76" s="4"/>
       <c r="J76" s="4"/>
-      <c r="K76" s="10"/>
-      <c r="L76" s="10"/>
-      <c r="M76" s="10"/>
-      <c r="N76" s="10"/>
+      <c r="K76" s="7"/>
+      <c r="L76" s="7"/>
+      <c r="M76" s="7"/>
+      <c r="N76" s="7"/>
     </row>
     <row r="77" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B77" s="20"/>
-      <c r="C77" s="12" t="s">
+      <c r="C77" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D77" s="10"/>
-      <c r="E77" s="10"/>
+      <c r="D77" s="7"/>
+      <c r="E77" s="7"/>
       <c r="F77" s="4"/>
       <c r="G77" s="4"/>
       <c r="H77" s="4"/>
       <c r="I77" s="4"/>
       <c r="J77" s="4"/>
-      <c r="K77" s="10">
+      <c r="K77" s="7">
         <f>D78</f>
         <v>3228.74</v>
       </c>
-      <c r="L77" s="10"/>
-      <c r="M77" s="10"/>
-      <c r="N77" s="10"/>
+      <c r="L77" s="7"/>
+      <c r="M77" s="7"/>
+      <c r="N77" s="7"/>
     </row>
     <row r="78" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B78" s="20"/>
-      <c r="C78" s="11" t="s">
+      <c r="C78" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="D78" s="10">
+      <c r="D78" s="7">
         <v>3228.74</v>
       </c>
-      <c r="E78" s="10">
+      <c r="E78" s="7">
         <f>D78</f>
         <v>3228.74</v>
       </c>
@@ -2703,92 +2703,86 @@
       <c r="H78" s="4"/>
       <c r="I78" s="4"/>
       <c r="J78" s="4"/>
-      <c r="K78" s="10"/>
-      <c r="L78" s="10"/>
-      <c r="M78" s="10"/>
-      <c r="N78" s="10"/>
+      <c r="K78" s="7"/>
+      <c r="L78" s="7"/>
+      <c r="M78" s="7"/>
+      <c r="N78" s="7"/>
     </row>
     <row r="79" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B79" s="21">
         <v>45047</v>
       </c>
-      <c r="C79" s="12" t="s">
+      <c r="C79" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D79" s="10"/>
-      <c r="E79" s="10"/>
+      <c r="D79" s="7"/>
+      <c r="E79" s="7"/>
       <c r="F79" s="4"/>
       <c r="G79" s="4"/>
       <c r="H79" s="4"/>
       <c r="I79" s="4"/>
       <c r="J79" s="4"/>
-      <c r="K79" s="10">
-        <f>D80</f>
-        <v>2441.4</v>
-      </c>
-      <c r="L79" s="10">
-        <f>D81</f>
-        <v>701.4</v>
-      </c>
-      <c r="M79" s="10"/>
-      <c r="N79" s="10"/>
+      <c r="K79" s="7">
+        <f>SUM(D80,(D82/2))</f>
+        <v>3937.6000000000004</v>
+      </c>
+      <c r="L79" s="7">
+        <f>SUM(D81,(D82/2))</f>
+        <v>2197.6</v>
+      </c>
+      <c r="M79" s="7"/>
+      <c r="N79" s="7"/>
     </row>
     <row r="80" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B80" s="21"/>
-      <c r="C80" s="11" t="s">
+      <c r="C80" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="D80" s="10">
+      <c r="D80" s="7">
         <f>2460-18.6</f>
         <v>2441.4</v>
       </c>
-      <c r="E80" s="10"/>
+      <c r="E80" s="7"/>
       <c r="F80" s="4"/>
       <c r="G80" s="4"/>
       <c r="H80" s="4"/>
       <c r="I80" s="4"/>
       <c r="J80" s="4"/>
-      <c r="K80" s="10">
-        <f>D82/2</f>
-        <v>1496.2</v>
-      </c>
-      <c r="L80" s="10">
-        <f>D82/2</f>
-        <v>1496.2</v>
-      </c>
-      <c r="M80" s="10"/>
-      <c r="N80" s="10"/>
+      <c r="K80" s="7"/>
+      <c r="L80" s="7"/>
+      <c r="M80" s="7"/>
+      <c r="N80" s="7"/>
     </row>
     <row r="81" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B81" s="21"/>
-      <c r="C81" s="11" t="s">
+      <c r="C81" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="D81" s="10">
+      <c r="D81" s="7">
         <f>720-18.6</f>
         <v>701.4</v>
       </c>
-      <c r="E81" s="10"/>
+      <c r="E81" s="7"/>
       <c r="F81" s="4"/>
       <c r="G81" s="4"/>
       <c r="H81" s="4"/>
       <c r="I81" s="4"/>
       <c r="J81" s="4"/>
-      <c r="K81" s="10"/>
-      <c r="L81" s="10"/>
-      <c r="M81" s="10"/>
-      <c r="N81" s="10"/>
+      <c r="K81" s="7"/>
+      <c r="L81" s="7"/>
+      <c r="M81" s="7"/>
+      <c r="N81" s="7"/>
     </row>
     <row r="82" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B82" s="21"/>
-      <c r="C82" s="11" t="s">
+      <c r="C82" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="D82" s="10">
+      <c r="D82" s="7">
         <f>3011-18.6</f>
         <v>2992.4</v>
       </c>
-      <c r="E82" s="10">
+      <c r="E82" s="7">
         <f>SUM(D80:D82)</f>
         <v>6135.2000000000007</v>
       </c>
@@ -2797,58 +2791,58 @@
       <c r="H82" s="4"/>
       <c r="I82" s="4"/>
       <c r="J82" s="4"/>
-      <c r="K82" s="10"/>
-      <c r="L82" s="10"/>
-      <c r="M82" s="10"/>
-      <c r="N82" s="10"/>
+      <c r="K82" s="7"/>
+      <c r="L82" s="7"/>
+      <c r="M82" s="7"/>
+      <c r="N82" s="7"/>
     </row>
     <row r="83" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B83" s="21"/>
       <c r="C83" s="4"/>
-      <c r="D83" s="10"/>
-      <c r="E83" s="10"/>
+      <c r="D83" s="7"/>
+      <c r="E83" s="7"/>
       <c r="F83" s="4"/>
       <c r="G83" s="4"/>
       <c r="H83" s="4"/>
       <c r="I83" s="4"/>
       <c r="J83" s="4"/>
-      <c r="K83" s="10"/>
-      <c r="L83" s="10"/>
-      <c r="M83" s="10"/>
-      <c r="N83" s="10"/>
+      <c r="K83" s="7"/>
+      <c r="L83" s="7"/>
+      <c r="M83" s="7"/>
+      <c r="N83" s="7"/>
     </row>
     <row r="84" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B84" s="21"/>
-      <c r="C84" s="12" t="s">
+      <c r="C84" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="D84" s="10"/>
-      <c r="E84" s="10"/>
+      <c r="D84" s="7"/>
+      <c r="E84" s="7"/>
       <c r="F84" s="4"/>
       <c r="G84" s="4"/>
       <c r="H84" s="4"/>
       <c r="I84" s="4"/>
       <c r="J84" s="4"/>
-      <c r="K84" s="10">
+      <c r="K84" s="7">
         <f>D85/2</f>
         <v>273.56</v>
       </c>
-      <c r="L84" s="10">
+      <c r="L84" s="7">
         <f>D85/2</f>
         <v>273.56</v>
       </c>
-      <c r="M84" s="10"/>
-      <c r="N84" s="10"/>
+      <c r="M84" s="7"/>
+      <c r="N84" s="7"/>
     </row>
     <row r="85" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B85" s="21"/>
-      <c r="C85" s="11" t="s">
+      <c r="C85" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D85" s="10">
+      <c r="D85" s="7">
         <v>547.12</v>
       </c>
-      <c r="E85" s="10">
+      <c r="E85" s="7">
         <f>D85</f>
         <v>547.12</v>
       </c>
@@ -2857,43 +2851,43 @@
       <c r="H85" s="4"/>
       <c r="I85" s="4"/>
       <c r="J85" s="4"/>
-      <c r="K85" s="10"/>
-      <c r="L85" s="10"/>
-      <c r="M85" s="10"/>
-      <c r="N85" s="10"/>
+      <c r="K85" s="7"/>
+      <c r="L85" s="7"/>
+      <c r="M85" s="7"/>
+      <c r="N85" s="7"/>
     </row>
     <row r="86" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B86" s="21"/>
-      <c r="C86" s="12" t="s">
+      <c r="C86" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="D86" s="10"/>
-      <c r="E86" s="10"/>
+      <c r="D86" s="7"/>
+      <c r="E86" s="7"/>
       <c r="F86" s="4"/>
       <c r="G86" s="4"/>
       <c r="H86" s="4"/>
       <c r="I86" s="4"/>
       <c r="J86" s="4"/>
-      <c r="K86" s="10">
+      <c r="K86" s="7">
         <f>D87/2</f>
         <v>172</v>
       </c>
-      <c r="L86" s="10">
+      <c r="L86" s="7">
         <f>D87/2</f>
         <v>172</v>
       </c>
-      <c r="M86" s="10"/>
-      <c r="N86" s="10"/>
+      <c r="M86" s="7"/>
+      <c r="N86" s="7"/>
     </row>
     <row r="87" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B87" s="21"/>
-      <c r="C87" s="11" t="s">
+      <c r="C87" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D87" s="10">
+      <c r="D87" s="7">
         <v>344</v>
       </c>
-      <c r="E87" s="10">
+      <c r="E87" s="7">
         <f>D87</f>
         <v>344</v>
       </c>
@@ -2902,62 +2896,62 @@
       <c r="H87" s="4"/>
       <c r="I87" s="4"/>
       <c r="J87" s="4"/>
-      <c r="K87" s="10"/>
-      <c r="L87" s="10"/>
-      <c r="M87" s="10"/>
-      <c r="N87" s="10"/>
+      <c r="K87" s="7"/>
+      <c r="L87" s="7"/>
+      <c r="M87" s="7"/>
+      <c r="N87" s="7"/>
     </row>
     <row r="88" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B88" s="21"/>
       <c r="C88" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D88" s="10"/>
-      <c r="E88" s="10"/>
+      <c r="D88" s="7"/>
+      <c r="E88" s="7"/>
       <c r="F88" s="4"/>
       <c r="G88" s="4"/>
       <c r="H88" s="4"/>
       <c r="I88" s="4"/>
       <c r="J88" s="4"/>
-      <c r="K88" s="10">
+      <c r="K88" s="7">
         <f>D90</f>
         <v>259</v>
       </c>
-      <c r="L88" s="10">
+      <c r="L88" s="7">
         <f>D89</f>
         <v>217</v>
       </c>
-      <c r="M88" s="10"/>
-      <c r="N88" s="10"/>
+      <c r="M88" s="7"/>
+      <c r="N88" s="7"/>
     </row>
     <row r="89" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B89" s="21"/>
-      <c r="C89" s="11" t="s">
+      <c r="C89" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="D89" s="10">
+      <c r="D89" s="7">
         <v>217</v>
       </c>
-      <c r="E89" s="10"/>
+      <c r="E89" s="7"/>
       <c r="F89" s="4"/>
       <c r="G89" s="4"/>
       <c r="H89" s="4"/>
       <c r="I89" s="4"/>
       <c r="J89" s="4"/>
-      <c r="K89" s="10"/>
-      <c r="L89" s="10"/>
-      <c r="M89" s="10"/>
-      <c r="N89" s="10"/>
+      <c r="K89" s="7"/>
+      <c r="L89" s="7"/>
+      <c r="M89" s="7"/>
+      <c r="N89" s="7"/>
     </row>
     <row r="90" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B90" s="21"/>
-      <c r="C90" s="11" t="s">
+      <c r="C90" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="D90" s="10">
+      <c r="D90" s="7">
         <v>259</v>
       </c>
-      <c r="E90" s="10">
+      <c r="E90" s="7">
         <f>SUM(D89:D90)</f>
         <v>476</v>
       </c>
@@ -2966,20 +2960,20 @@
       <c r="H90" s="4"/>
       <c r="I90" s="4"/>
       <c r="J90" s="4"/>
-      <c r="K90" s="10"/>
-      <c r="L90" s="10"/>
-      <c r="M90" s="10"/>
-      <c r="N90" s="10"/>
+      <c r="K90" s="7"/>
+      <c r="L90" s="7"/>
+      <c r="M90" s="7"/>
+      <c r="N90" s="7"/>
     </row>
     <row r="91" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B91" s="22" t="s">
+      <c r="B91" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="C91" s="12" t="s">
+      <c r="C91" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="D91" s="10"/>
-      <c r="E91" s="10">
+      <c r="D91" s="7"/>
+      <c r="E91" s="7">
         <f>D92</f>
         <v>2774</v>
       </c>
@@ -2988,43 +2982,43 @@
       <c r="H91" s="4"/>
       <c r="I91" s="4"/>
       <c r="J91" s="4"/>
-      <c r="K91" s="10">
+      <c r="K91" s="7">
         <f>D92</f>
         <v>2774</v>
       </c>
-      <c r="L91" s="10">
+      <c r="L91" s="7">
         <f>D92</f>
         <v>2774</v>
       </c>
-      <c r="M91" s="10"/>
-      <c r="N91" s="10"/>
+      <c r="M91" s="7"/>
+      <c r="N91" s="7"/>
     </row>
     <row r="92" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B92" s="22"/>
-      <c r="C92" s="11" t="s">
+      <c r="B92" s="13"/>
+      <c r="C92" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="D92" s="10">
+      <c r="D92" s="7">
         <v>2774</v>
       </c>
-      <c r="E92" s="10"/>
+      <c r="E92" s="7"/>
       <c r="F92" s="4"/>
       <c r="G92" s="4"/>
       <c r="H92" s="4"/>
       <c r="I92" s="4"/>
       <c r="J92" s="4"/>
-      <c r="K92" s="10"/>
-      <c r="L92" s="10"/>
-      <c r="M92" s="10"/>
-      <c r="N92" s="10"/>
+      <c r="K92" s="7"/>
+      <c r="L92" s="7"/>
+      <c r="M92" s="7"/>
+      <c r="N92" s="7"/>
     </row>
     <row r="93" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B93" s="22"/>
-      <c r="C93" s="12" t="s">
+      <c r="B93" s="13"/>
+      <c r="C93" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="D93" s="10"/>
-      <c r="E93" s="10">
+      <c r="D93" s="7"/>
+      <c r="E93" s="7">
         <f>D94</f>
         <v>5891</v>
       </c>
@@ -3033,43 +3027,43 @@
       <c r="H93" s="4"/>
       <c r="I93" s="4"/>
       <c r="J93" s="4"/>
-      <c r="K93" s="10">
+      <c r="K93" s="7">
         <f>D94</f>
         <v>5891</v>
       </c>
-      <c r="L93" s="10">
+      <c r="L93" s="7">
         <f>D94</f>
         <v>5891</v>
       </c>
-      <c r="M93" s="10"/>
-      <c r="N93" s="10"/>
+      <c r="M93" s="7"/>
+      <c r="N93" s="7"/>
     </row>
     <row r="94" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B94" s="22"/>
-      <c r="C94" s="11" t="s">
+      <c r="B94" s="13"/>
+      <c r="C94" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="D94" s="10">
+      <c r="D94" s="7">
         <v>5891</v>
       </c>
-      <c r="E94" s="10"/>
+      <c r="E94" s="7"/>
       <c r="F94" s="4"/>
       <c r="G94" s="4"/>
       <c r="H94" s="4"/>
       <c r="I94" s="4"/>
       <c r="J94" s="4"/>
-      <c r="K94" s="10"/>
-      <c r="L94" s="10"/>
-      <c r="M94" s="10"/>
-      <c r="N94" s="10"/>
+      <c r="K94" s="7"/>
+      <c r="L94" s="7"/>
+      <c r="M94" s="7"/>
+      <c r="N94" s="7"/>
     </row>
     <row r="95" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B95" s="22"/>
-      <c r="C95" s="12" t="s">
+      <c r="B95" s="13"/>
+      <c r="C95" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="D95" s="10"/>
-      <c r="E95" s="10">
+      <c r="D95" s="7"/>
+      <c r="E95" s="7">
         <f>D96</f>
         <v>5893</v>
       </c>
@@ -3078,35 +3072,35 @@
       <c r="H95" s="4"/>
       <c r="I95" s="4"/>
       <c r="J95" s="4"/>
-      <c r="K95" s="10">
+      <c r="K95" s="7">
         <f>D96</f>
         <v>5893</v>
       </c>
-      <c r="L95" s="10">
+      <c r="L95" s="7">
         <f>D96</f>
         <v>5893</v>
       </c>
-      <c r="M95" s="10"/>
-      <c r="N95" s="10"/>
+      <c r="M95" s="7"/>
+      <c r="N95" s="7"/>
     </row>
     <row r="96" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B96" s="22"/>
-      <c r="C96" s="11" t="s">
+      <c r="B96" s="13"/>
+      <c r="C96" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="D96" s="10">
+      <c r="D96" s="7">
         <v>5893</v>
       </c>
-      <c r="E96" s="10"/>
+      <c r="E96" s="7"/>
       <c r="F96" s="4"/>
       <c r="G96" s="4"/>
       <c r="H96" s="4"/>
       <c r="I96" s="4"/>
       <c r="J96" s="4"/>
-      <c r="K96" s="10"/>
-      <c r="L96" s="10"/>
-      <c r="M96" s="10"/>
-      <c r="N96" s="10"/>
+      <c r="K96" s="7"/>
+      <c r="L96" s="7"/>
+      <c r="M96" s="7"/>
+      <c r="N96" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -3124,5 +3118,8 @@
     <mergeCell ref="B58:B64"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;"Aptos"&amp;12&amp;KFF8C00 CONFIDENTIAL&amp;1#_x000D_</oddHeader>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Japan expense spreadsheet and add utility scripts
</commit_message>
<xml_diff>
--- a/JAPAN EXPENSE.xlsx
+++ b/JAPAN EXPENSE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amadeusworkplace-my.sharepoint.com/personal/jonjester_reguyal_amadeus_com/Documents/Desktop/JAPAN TRIP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="323" documentId="8_{8DD0C82D-92A8-469F-8A5F-7373CA3C28E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9DD11E7-D0D2-453E-80C7-D40C08B12024}"/>
+  <xr:revisionPtr revIDLastSave="368" documentId="8_{8DD0C82D-92A8-469F-8A5F-7373CA3C28E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0425E365-0358-4AA7-ACA8-DC7E48A7E1CC}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{77262E9F-01AC-4670-AAC1-0C05B2A698AE}"/>
+    <workbookView xWindow="-30828" yWindow="-2916" windowWidth="30936" windowHeight="16776" xr2:uid="{77262E9F-01AC-4670-AAC1-0C05B2A698AE}"/>
   </bookViews>
   <sheets>
     <sheet name="Japan Trip" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="94">
   <si>
     <t xml:space="preserve">FLIGHT </t>
   </si>
@@ -309,6 +309,18 @@
   </si>
   <si>
     <t xml:space="preserve">jes kape </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travel INSURANCE </t>
+  </si>
+  <si>
+    <t>Grab to airport and home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grab Home to Airport </t>
+  </si>
+  <si>
+    <t>JAPAN VISA</t>
   </si>
 </sst>
 </file>
@@ -404,7 +416,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -490,12 +502,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -522,9 +545,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -563,6 +583,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -904,23 +939,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{228C58C2-89C8-422F-BB16-5EF3E8507030}">
-  <dimension ref="B1:W96"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B1:W100"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="8.88671875" style="11"/>
-    <col min="3" max="3" width="31.109375" customWidth="1"/>
-    <col min="4" max="5" width="10.44140625" style="1" customWidth="1"/>
-    <col min="6" max="10" width="8.88671875" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="19.88671875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="21.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" style="11"/>
+    <col min="3" max="3" width="31.140625" customWidth="1"/>
+    <col min="4" max="5" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="10" width="8.85546875" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="19.85546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="21.7109375" style="1" customWidth="1"/>
     <col min="13" max="13" width="13" style="1" customWidth="1"/>
-    <col min="14" max="14" width="15.5546875" style="1" customWidth="1"/>
-    <col min="19" max="19" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.5703125" style="1" customWidth="1"/>
+    <col min="19" max="19" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="8.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:23" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B1" s="10" t="s">
         <v>9</v>
       </c>
@@ -951,8 +987,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B2" s="22">
+    <row r="2" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B2" s="21">
         <v>42491</v>
       </c>
       <c r="C2" s="4" t="s">
@@ -976,8 +1012,8 @@
       <c r="M2" s="7"/>
       <c r="N2" s="7"/>
     </row>
-    <row r="3" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B3" s="22"/>
+    <row r="3" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B3" s="21"/>
       <c r="C3" s="8" t="s">
         <v>32</v>
       </c>
@@ -998,8 +1034,8 @@
       <c r="M3" s="7"/>
       <c r="N3" s="7"/>
     </row>
-    <row r="4" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B4" s="22"/>
+    <row r="4" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B4" s="21"/>
       <c r="C4" s="4" t="s">
         <v>7</v>
       </c>
@@ -1021,8 +1057,8 @@
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
     </row>
-    <row r="5" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B5" s="22"/>
+    <row r="5" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B5" s="21"/>
       <c r="C5" s="8" t="s">
         <v>32</v>
       </c>
@@ -1044,8 +1080,8 @@
       <c r="M5" s="7"/>
       <c r="N5" s="7"/>
     </row>
-    <row r="6" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B6" s="22"/>
+    <row r="6" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B6" s="21"/>
       <c r="C6" s="4" t="s">
         <v>6</v>
       </c>
@@ -1073,8 +1109,8 @@
         <v>1161</v>
       </c>
     </row>
-    <row r="7" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B7" s="22"/>
+    <row r="7" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B7" s="21"/>
       <c r="C7" s="8" t="s">
         <v>38</v>
       </c>
@@ -1096,8 +1132,8 @@
       <c r="M7" s="7"/>
       <c r="N7" s="7"/>
     </row>
-    <row r="8" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B8" s="22"/>
+    <row r="8" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B8" s="21"/>
       <c r="C8" s="4" t="s">
         <v>5</v>
       </c>
@@ -1124,7 +1160,7 @@
         <f>D9/4</f>
         <v>1158</v>
       </c>
-      <c r="S8" s="14" t="s">
+      <c r="S8" s="13" t="s">
         <v>75</v>
       </c>
       <c r="T8" s="2" t="s">
@@ -1140,8 +1176,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B9" s="22"/>
+    <row r="9" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B9" s="21"/>
       <c r="C9" s="8" t="s">
         <v>38</v>
       </c>
@@ -1162,20 +1198,20 @@
       <c r="L9" s="7"/>
       <c r="M9" s="7"/>
       <c r="N9" s="7"/>
-      <c r="S9" s="15"/>
+      <c r="S9" s="14"/>
       <c r="T9" s="3">
-        <f>SUM(K2:K96)</f>
-        <v>78934.909999999974</v>
+        <f>SUM(K2:K100)</f>
+        <v>84847.909999999974</v>
       </c>
       <c r="U9" s="3">
-        <f>SUM(L2:L96)</f>
-        <v>65613.739999999991</v>
+        <f>SUM(L2:L100)</f>
+        <v>71526.739999999991</v>
       </c>
       <c r="V9" s="4"/>
       <c r="W9" s="4"/>
     </row>
-    <row r="10" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B10" s="22"/>
+    <row r="10" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B10" s="21"/>
       <c r="C10" s="4" t="s">
         <v>8</v>
       </c>
@@ -1202,14 +1238,14 @@
         <f>D11/4</f>
         <v>256</v>
       </c>
-      <c r="S10" s="16"/>
-      <c r="T10" s="17"/>
-      <c r="U10" s="17"/>
-      <c r="V10" s="17"/>
-      <c r="W10" s="18"/>
-    </row>
-    <row r="11" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B11" s="22"/>
+      <c r="S10" s="15"/>
+      <c r="T10" s="16"/>
+      <c r="U10" s="16"/>
+      <c r="V10" s="16"/>
+      <c r="W10" s="17"/>
+    </row>
+    <row r="11" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B11" s="21"/>
       <c r="C11" s="4"/>
       <c r="D11" s="7">
         <f>256*4</f>
@@ -1241,8 +1277,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B12" s="22"/>
+    <row r="12" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B12" s="21"/>
       <c r="C12" s="4" t="s">
         <v>11</v>
       </c>
@@ -1284,8 +1320,8 @@
         <v>714.91500000000008</v>
       </c>
     </row>
-    <row r="13" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B13" s="22"/>
+    <row r="13" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B13" s="21"/>
       <c r="C13" s="8" t="s">
         <v>32</v>
       </c>
@@ -1302,14 +1338,14 @@
       <c r="L13" s="7"/>
       <c r="M13" s="7"/>
       <c r="N13" s="7"/>
-      <c r="S13" s="16"/>
-      <c r="T13" s="17"/>
-      <c r="U13" s="17"/>
-      <c r="V13" s="17"/>
-      <c r="W13" s="18"/>
-    </row>
-    <row r="14" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B14" s="23">
+      <c r="S13" s="15"/>
+      <c r="T13" s="16"/>
+      <c r="U13" s="16"/>
+      <c r="V13" s="16"/>
+      <c r="W13" s="17"/>
+    </row>
+    <row r="14" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B14" s="22">
         <v>42856</v>
       </c>
       <c r="C14" s="4" t="s">
@@ -1348,8 +1384,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B15" s="23"/>
+    <row r="15" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B15" s="22"/>
       <c r="C15" s="8" t="s">
         <v>30</v>
       </c>
@@ -1384,8 +1420,8 @@
       </c>
       <c r="W15" s="4"/>
     </row>
-    <row r="16" spans="2:23" x14ac:dyDescent="0.3">
-      <c r="B16" s="23"/>
+    <row r="16" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B16" s="22"/>
       <c r="C16" s="4" t="s">
         <v>12</v>
       </c>
@@ -1407,8 +1443,8 @@
       <c r="M16" s="7"/>
       <c r="N16" s="7"/>
     </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B17" s="23"/>
+    <row r="17" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B17" s="22"/>
       <c r="C17" s="8" t="s">
         <v>36</v>
       </c>
@@ -1426,8 +1462,8 @@
       <c r="M17" s="7"/>
       <c r="N17" s="7"/>
     </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B18" s="23"/>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B18" s="22"/>
       <c r="C18" s="8" t="s">
         <v>37</v>
       </c>
@@ -1445,8 +1481,8 @@
       <c r="M18" s="7"/>
       <c r="N18" s="7"/>
     </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B19" s="23"/>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B19" s="22"/>
       <c r="C19" s="4" t="s">
         <v>13</v>
       </c>
@@ -1465,8 +1501,8 @@
       <c r="M19" s="7"/>
       <c r="N19" s="7"/>
     </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B20" s="23"/>
+    <row r="20" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B20" s="22"/>
       <c r="C20" s="8" t="s">
         <v>35</v>
       </c>
@@ -1484,8 +1520,8 @@
       <c r="M20" s="7"/>
       <c r="N20" s="7"/>
     </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B21" s="23"/>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B21" s="22"/>
       <c r="C21" s="4" t="s">
         <v>14</v>
       </c>
@@ -1507,8 +1543,8 @@
       <c r="M21" s="7"/>
       <c r="N21" s="7"/>
     </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B22" s="23"/>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B22" s="22"/>
       <c r="C22" s="8" t="s">
         <v>89</v>
       </c>
@@ -1527,8 +1563,8 @@
       <c r="M22" s="7"/>
       <c r="N22" s="7"/>
     </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B23" s="23"/>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B23" s="22"/>
       <c r="C23" s="8" t="s">
         <v>34</v>
       </c>
@@ -1550,8 +1586,8 @@
       <c r="M23" s="7"/>
       <c r="N23" s="7"/>
     </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B24" s="23"/>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B24" s="22"/>
       <c r="C24" s="4" t="s">
         <v>15</v>
       </c>
@@ -1570,8 +1606,8 @@
       <c r="M24" s="7"/>
       <c r="N24" s="7"/>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B25" s="23"/>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B25" s="22"/>
       <c r="C25" s="8" t="s">
         <v>33</v>
       </c>
@@ -1589,8 +1625,8 @@
       <c r="M25" s="7"/>
       <c r="N25" s="7"/>
     </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B26" s="23"/>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B26" s="22"/>
       <c r="C26" s="4" t="s">
         <v>16</v>
       </c>
@@ -1612,8 +1648,8 @@
       <c r="M26" s="7"/>
       <c r="N26" s="7"/>
     </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B27" s="23"/>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B27" s="22"/>
       <c r="C27" s="8" t="s">
         <v>30</v>
       </c>
@@ -1631,8 +1667,8 @@
       <c r="M27" s="7"/>
       <c r="N27" s="7"/>
     </row>
-    <row r="28" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B28" s="23"/>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B28" s="22"/>
       <c r="C28" s="8" t="s">
         <v>31</v>
       </c>
@@ -1650,8 +1686,8 @@
       <c r="M28" s="7"/>
       <c r="N28" s="7"/>
     </row>
-    <row r="29" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B29" s="23"/>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B29" s="22"/>
       <c r="C29" s="4" t="s">
         <v>17</v>
       </c>
@@ -1673,8 +1709,8 @@
       <c r="M29" s="7"/>
       <c r="N29" s="7"/>
     </row>
-    <row r="30" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B30" s="23"/>
+    <row r="30" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B30" s="22"/>
       <c r="C30" s="8" t="s">
         <v>32</v>
       </c>
@@ -1692,8 +1728,8 @@
       <c r="M30" s="7"/>
       <c r="N30" s="7"/>
     </row>
-    <row r="31" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B31" s="23"/>
+    <row r="31" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B31" s="22"/>
       <c r="C31" s="4" t="s">
         <v>18</v>
       </c>
@@ -1715,8 +1751,8 @@
       <c r="M31" s="7"/>
       <c r="N31" s="7"/>
     </row>
-    <row r="32" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B32" s="23"/>
+    <row r="32" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B32" s="22"/>
       <c r="C32" s="8" t="s">
         <v>30</v>
       </c>
@@ -1735,8 +1771,8 @@
       <c r="M32" s="7"/>
       <c r="N32" s="7"/>
     </row>
-    <row r="33" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B33" s="23"/>
+    <row r="33" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B33" s="22"/>
       <c r="C33" s="8" t="s">
         <v>31</v>
       </c>
@@ -1758,8 +1794,8 @@
       <c r="M33" s="7"/>
       <c r="N33" s="7"/>
     </row>
-    <row r="34" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B34" s="23"/>
+    <row r="34" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B34" s="22"/>
       <c r="C34" s="4" t="s">
         <v>19</v>
       </c>
@@ -1784,8 +1820,8 @@
         <v>386.09000000000003</v>
       </c>
     </row>
-    <row r="35" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B35" s="23"/>
+    <row r="35" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B35" s="22"/>
       <c r="C35" s="8" t="s">
         <v>27</v>
       </c>
@@ -1804,8 +1840,8 @@
       <c r="M35" s="7"/>
       <c r="N35" s="7"/>
     </row>
-    <row r="36" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B36" s="23"/>
+    <row r="36" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B36" s="22"/>
       <c r="C36" s="8" t="s">
         <v>28</v>
       </c>
@@ -1824,8 +1860,8 @@
       <c r="M36" s="7"/>
       <c r="N36" s="7"/>
     </row>
-    <row r="37" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B37" s="23"/>
+    <row r="37" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B37" s="22"/>
       <c r="C37" s="8" t="s">
         <v>29</v>
       </c>
@@ -1846,8 +1882,8 @@
       <c r="M37" s="7"/>
       <c r="N37" s="7"/>
     </row>
-    <row r="38" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B38" s="24">
+    <row r="38" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B38" s="23">
         <v>43221</v>
       </c>
       <c r="C38" s="4" t="s">
@@ -1871,8 +1907,8 @@
       <c r="M38" s="7"/>
       <c r="N38" s="7"/>
     </row>
-    <row r="39" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B39" s="24"/>
+    <row r="39" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B39" s="23"/>
       <c r="C39" s="8" t="s">
         <v>87</v>
       </c>
@@ -1890,8 +1926,8 @@
       <c r="M39" s="7"/>
       <c r="N39" s="7"/>
     </row>
-    <row r="40" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B40" s="25">
+    <row r="40" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B40" s="24">
         <v>43586</v>
       </c>
       <c r="C40" s="4" t="s">
@@ -1912,8 +1948,8 @@
       <c r="M40" s="7"/>
       <c r="N40" s="7"/>
     </row>
-    <row r="41" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B41" s="25"/>
+    <row r="41" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B41" s="24"/>
       <c r="C41" s="8" t="s">
         <v>88</v>
       </c>
@@ -1931,8 +1967,8 @@
       <c r="M41" s="7"/>
       <c r="N41" s="7"/>
     </row>
-    <row r="42" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B42" s="25"/>
+    <row r="42" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B42" s="24"/>
       <c r="C42" s="4" t="s">
         <v>22</v>
       </c>
@@ -1957,8 +1993,8 @@
         <v>78</v>
       </c>
     </row>
-    <row r="43" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B43" s="25"/>
+    <row r="43" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B43" s="24"/>
       <c r="C43" s="8" t="s">
         <v>26</v>
       </c>
@@ -1976,8 +2012,8 @@
       <c r="M43" s="7"/>
       <c r="N43" s="7"/>
     </row>
-    <row r="44" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B44" s="25"/>
+    <row r="44" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B44" s="24"/>
       <c r="C44" s="8" t="s">
         <v>1</v>
       </c>
@@ -1995,8 +2031,8 @@
       <c r="M44" s="7"/>
       <c r="N44" s="7"/>
     </row>
-    <row r="45" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B45" s="25"/>
+    <row r="45" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B45" s="24"/>
       <c r="C45" s="8" t="s">
         <v>4</v>
       </c>
@@ -2014,8 +2050,8 @@
       <c r="M45" s="7"/>
       <c r="N45" s="7"/>
     </row>
-    <row r="46" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B46" s="25"/>
+    <row r="46" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B46" s="24"/>
       <c r="C46" s="4" t="s">
         <v>23</v>
       </c>
@@ -2037,8 +2073,8 @@
       <c r="M46" s="7"/>
       <c r="N46" s="7"/>
     </row>
-    <row r="47" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B47" s="25"/>
+    <row r="47" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B47" s="24"/>
       <c r="C47" s="8" t="s">
         <v>39</v>
       </c>
@@ -2056,8 +2092,8 @@
       <c r="M47" s="7"/>
       <c r="N47" s="7"/>
     </row>
-    <row r="48" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B48" s="25"/>
+    <row r="48" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B48" s="24"/>
       <c r="C48" s="4" t="s">
         <v>24</v>
       </c>
@@ -2073,8 +2109,8 @@
       <c r="M48" s="7"/>
       <c r="N48" s="7"/>
     </row>
-    <row r="49" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B49" s="25"/>
+    <row r="49" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B49" s="24"/>
       <c r="C49" s="8" t="s">
         <v>40</v>
       </c>
@@ -2105,8 +2141,8 @@
         <v>250.82500000000002</v>
       </c>
     </row>
-    <row r="50" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B50" s="25"/>
+    <row r="50" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B50" s="24"/>
       <c r="C50" s="8" t="s">
         <v>42</v>
       </c>
@@ -2125,8 +2161,8 @@
       <c r="M50" s="7"/>
       <c r="N50" s="7"/>
     </row>
-    <row r="51" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B51" s="25"/>
+    <row r="51" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B51" s="24"/>
       <c r="C51" s="8" t="s">
         <v>41</v>
       </c>
@@ -2145,8 +2181,8 @@
       <c r="M51" s="7"/>
       <c r="N51" s="7"/>
     </row>
-    <row r="52" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B52" s="25"/>
+    <row r="52" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B52" s="24"/>
       <c r="C52" s="8" t="s">
         <v>43</v>
       </c>
@@ -2168,8 +2204,8 @@
       <c r="M52" s="7"/>
       <c r="N52" s="7"/>
     </row>
-    <row r="53" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B53" s="25"/>
+    <row r="53" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B53" s="24"/>
       <c r="C53" s="4" t="s">
         <v>25</v>
       </c>
@@ -2188,8 +2224,8 @@
       <c r="M53" s="7"/>
       <c r="N53" s="7"/>
     </row>
-    <row r="54" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B54" s="25"/>
+    <row r="54" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B54" s="24"/>
       <c r="C54" s="8" t="s">
         <v>44</v>
       </c>
@@ -2207,8 +2243,8 @@
       <c r="M54" s="7"/>
       <c r="N54" s="7"/>
     </row>
-    <row r="55" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B55" s="25"/>
+    <row r="55" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B55" s="24"/>
       <c r="C55" s="9" t="s">
         <v>45</v>
       </c>
@@ -2230,8 +2266,8 @@
       <c r="M55" s="7"/>
       <c r="N55" s="7"/>
     </row>
-    <row r="56" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B56" s="25"/>
+    <row r="56" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B56" s="24"/>
       <c r="C56" s="8" t="s">
         <v>2</v>
       </c>
@@ -2249,8 +2285,8 @@
       <c r="M56" s="7"/>
       <c r="N56" s="7"/>
     </row>
-    <row r="57" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B57" s="25"/>
+    <row r="57" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B57" s="24"/>
       <c r="C57" s="8" t="s">
         <v>1</v>
       </c>
@@ -2270,8 +2306,8 @@
       <c r="M57" s="7"/>
       <c r="N57" s="7"/>
     </row>
-    <row r="58" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B58" s="26">
+    <row r="58" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B58" s="25">
         <v>43952</v>
       </c>
       <c r="C58" s="9" t="s">
@@ -2292,8 +2328,8 @@
       <c r="M58" s="7"/>
       <c r="N58" s="7"/>
     </row>
-    <row r="59" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B59" s="26"/>
+    <row r="59" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B59" s="25"/>
       <c r="C59" s="8" t="s">
         <v>48</v>
       </c>
@@ -2311,8 +2347,8 @@
       <c r="M59" s="7"/>
       <c r="N59" s="7"/>
     </row>
-    <row r="60" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B60" s="26"/>
+    <row r="60" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B60" s="25"/>
       <c r="C60" s="9" t="s">
         <v>49</v>
       </c>
@@ -2334,8 +2370,8 @@
       <c r="M60" s="7"/>
       <c r="N60" s="7"/>
     </row>
-    <row r="61" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B61" s="26"/>
+    <row r="61" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B61" s="25"/>
       <c r="C61" s="8" t="s">
         <v>50</v>
       </c>
@@ -2353,8 +2389,8 @@
       <c r="M61" s="7"/>
       <c r="N61" s="7"/>
     </row>
-    <row r="62" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B62" s="26"/>
+    <row r="62" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B62" s="25"/>
       <c r="C62" s="9" t="s">
         <v>51</v>
       </c>
@@ -2376,8 +2412,8 @@
       <c r="M62" s="7"/>
       <c r="N62" s="7"/>
     </row>
-    <row r="63" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B63" s="26"/>
+    <row r="63" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B63" s="25"/>
       <c r="C63" s="8" t="s">
         <v>52</v>
       </c>
@@ -2396,8 +2432,8 @@
       <c r="M63" s="7"/>
       <c r="N63" s="7"/>
     </row>
-    <row r="64" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B64" s="26"/>
+    <row r="64" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B64" s="25"/>
       <c r="C64" s="8" t="s">
         <v>53</v>
       </c>
@@ -2418,8 +2454,8 @@
       <c r="M64" s="7"/>
       <c r="N64" s="7"/>
     </row>
-    <row r="65" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B65" s="19">
+    <row r="65" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B65" s="18">
         <v>44317</v>
       </c>
       <c r="C65" s="9" t="s">
@@ -2440,8 +2476,8 @@
       <c r="M65" s="7"/>
       <c r="N65" s="7"/>
     </row>
-    <row r="66" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B66" s="19"/>
+    <row r="66" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B66" s="18"/>
       <c r="C66" s="8" t="s">
         <v>55</v>
       </c>
@@ -2459,8 +2495,8 @@
       <c r="M66" s="7"/>
       <c r="N66" s="7"/>
     </row>
-    <row r="67" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B67" s="19"/>
+    <row r="67" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B67" s="18"/>
       <c r="C67" s="9" t="s">
         <v>10</v>
       </c>
@@ -2485,8 +2521,8 @@
       </c>
       <c r="N67" s="7"/>
     </row>
-    <row r="68" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B68" s="19"/>
+    <row r="68" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B68" s="18"/>
       <c r="C68" s="8" t="s">
         <v>56</v>
       </c>
@@ -2504,8 +2540,8 @@
       <c r="M68" s="7"/>
       <c r="N68" s="7"/>
     </row>
-    <row r="69" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B69" s="20">
+    <row r="69" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B69" s="19">
         <v>44682</v>
       </c>
       <c r="C69" s="9" t="s">
@@ -2529,8 +2565,8 @@
       <c r="M69" s="7"/>
       <c r="N69" s="7"/>
     </row>
-    <row r="70" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B70" s="20"/>
+    <row r="70" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B70" s="19"/>
       <c r="C70" s="8" t="s">
         <v>58</v>
       </c>
@@ -2549,8 +2585,8 @@
       <c r="M70" s="7"/>
       <c r="N70" s="7"/>
     </row>
-    <row r="71" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B71" s="20"/>
+    <row r="71" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B71" s="19"/>
       <c r="C71" s="8" t="s">
         <v>59</v>
       </c>
@@ -2571,8 +2607,8 @@
       <c r="M71" s="7"/>
       <c r="N71" s="7"/>
     </row>
-    <row r="72" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B72" s="20"/>
+    <row r="72" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B72" s="19"/>
       <c r="C72" s="9" t="s">
         <v>60</v>
       </c>
@@ -2594,8 +2630,8 @@
       <c r="M72" s="7"/>
       <c r="N72" s="7"/>
     </row>
-    <row r="73" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B73" s="20"/>
+    <row r="73" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B73" s="19"/>
       <c r="C73" s="8" t="s">
         <v>61</v>
       </c>
@@ -2613,8 +2649,8 @@
       <c r="M73" s="7"/>
       <c r="N73" s="7"/>
     </row>
-    <row r="74" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B74" s="20"/>
+    <row r="74" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B74" s="19"/>
       <c r="C74" s="8" t="s">
         <v>62</v>
       </c>
@@ -2635,8 +2671,8 @@
       <c r="M74" s="7"/>
       <c r="N74" s="7"/>
     </row>
-    <row r="75" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B75" s="20"/>
+    <row r="75" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B75" s="19"/>
       <c r="C75" s="8" t="s">
         <v>63</v>
       </c>
@@ -2658,8 +2694,8 @@
       <c r="M75" s="7"/>
       <c r="N75" s="7"/>
     </row>
-    <row r="76" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B76" s="20"/>
+    <row r="76" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B76" s="19"/>
       <c r="C76" s="8" t="s">
         <v>64</v>
       </c>
@@ -2680,8 +2716,8 @@
       <c r="M76" s="7"/>
       <c r="N76" s="7"/>
     </row>
-    <row r="77" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B77" s="20"/>
+    <row r="77" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B77" s="19"/>
       <c r="C77" s="9" t="s">
         <v>65</v>
       </c>
@@ -2700,8 +2736,8 @@
       <c r="M77" s="7"/>
       <c r="N77" s="7"/>
     </row>
-    <row r="78" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B78" s="20"/>
+    <row r="78" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B78" s="19"/>
       <c r="C78" s="8" t="s">
         <v>66</v>
       </c>
@@ -2722,8 +2758,8 @@
       <c r="M78" s="7"/>
       <c r="N78" s="7"/>
     </row>
-    <row r="79" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B79" s="21">
+    <row r="79" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B79" s="20">
         <v>45047</v>
       </c>
       <c r="C79" s="9" t="s">
@@ -2747,8 +2783,8 @@
       <c r="M79" s="7"/>
       <c r="N79" s="7"/>
     </row>
-    <row r="80" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B80" s="21"/>
+    <row r="80" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B80" s="20"/>
       <c r="C80" s="8" t="s">
         <v>68</v>
       </c>
@@ -2767,8 +2803,8 @@
       <c r="M80" s="7"/>
       <c r="N80" s="7"/>
     </row>
-    <row r="81" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B81" s="21"/>
+    <row r="81" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B81" s="20"/>
       <c r="C81" s="8" t="s">
         <v>69</v>
       </c>
@@ -2787,8 +2823,8 @@
       <c r="M81" s="7"/>
       <c r="N81" s="7"/>
     </row>
-    <row r="82" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B82" s="21"/>
+    <row r="82" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B82" s="20"/>
       <c r="C82" s="8" t="s">
         <v>70</v>
       </c>
@@ -2810,8 +2846,8 @@
       <c r="M82" s="7"/>
       <c r="N82" s="7"/>
     </row>
-    <row r="83" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B83" s="21"/>
+    <row r="83" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B83" s="20"/>
       <c r="C83" s="4"/>
       <c r="D83" s="7"/>
       <c r="E83" s="7"/>
@@ -2825,8 +2861,8 @@
       <c r="M83" s="7"/>
       <c r="N83" s="7"/>
     </row>
-    <row r="84" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B84" s="21"/>
+    <row r="84" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B84" s="20"/>
       <c r="C84" s="9" t="s">
         <v>71</v>
       </c>
@@ -2848,8 +2884,8 @@
       <c r="M84" s="7"/>
       <c r="N84" s="7"/>
     </row>
-    <row r="85" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B85" s="21"/>
+    <row r="85" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B85" s="20"/>
       <c r="C85" s="8" t="s">
         <v>32</v>
       </c>
@@ -2870,8 +2906,8 @@
       <c r="M85" s="7"/>
       <c r="N85" s="7"/>
     </row>
-    <row r="86" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B86" s="21"/>
+    <row r="86" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B86" s="20"/>
       <c r="C86" s="9" t="s">
         <v>72</v>
       </c>
@@ -2893,8 +2929,8 @@
       <c r="M86" s="7"/>
       <c r="N86" s="7"/>
     </row>
-    <row r="87" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B87" s="21"/>
+    <row r="87" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B87" s="20"/>
       <c r="C87" s="8" t="s">
         <v>32</v>
       </c>
@@ -2915,8 +2951,8 @@
       <c r="M87" s="7"/>
       <c r="N87" s="7"/>
     </row>
-    <row r="88" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B88" s="21"/>
+    <row r="88" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B88" s="20"/>
       <c r="C88" s="4" t="s">
         <v>73</v>
       </c>
@@ -2938,8 +2974,8 @@
       <c r="M88" s="7"/>
       <c r="N88" s="7"/>
     </row>
-    <row r="89" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B89" s="21"/>
+    <row r="89" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B89" s="20"/>
       <c r="C89" s="8" t="s">
         <v>69</v>
       </c>
@@ -2957,8 +2993,8 @@
       <c r="M89" s="7"/>
       <c r="N89" s="7"/>
     </row>
-    <row r="90" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B90" s="21"/>
+    <row r="90" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B90" s="20"/>
       <c r="C90" s="8" t="s">
         <v>74</v>
       </c>
@@ -2979,8 +3015,8 @@
       <c r="M90" s="7"/>
       <c r="N90" s="7"/>
     </row>
-    <row r="91" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B91" s="13" t="s">
+    <row r="91" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B91" s="28" t="s">
         <v>81</v>
       </c>
       <c r="C91" s="9" t="s">
@@ -3007,8 +3043,8 @@
       <c r="M91" s="7"/>
       <c r="N91" s="7"/>
     </row>
-    <row r="92" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B92" s="13"/>
+    <row r="92" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B92" s="29"/>
       <c r="C92" s="8" t="s">
         <v>83</v>
       </c>
@@ -3026,8 +3062,8 @@
       <c r="M92" s="7"/>
       <c r="N92" s="7"/>
     </row>
-    <row r="93" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B93" s="13"/>
+    <row r="93" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B93" s="29"/>
       <c r="C93" s="9" t="s">
         <v>84</v>
       </c>
@@ -3052,8 +3088,8 @@
       <c r="M93" s="7"/>
       <c r="N93" s="7"/>
     </row>
-    <row r="94" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B94" s="13"/>
+    <row r="94" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B94" s="29"/>
       <c r="C94" s="8" t="s">
         <v>83</v>
       </c>
@@ -3071,8 +3107,8 @@
       <c r="M94" s="7"/>
       <c r="N94" s="7"/>
     </row>
-    <row r="95" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B95" s="13"/>
+    <row r="95" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B95" s="29"/>
       <c r="C95" s="9" t="s">
         <v>85</v>
       </c>
@@ -3097,8 +3133,8 @@
       <c r="M95" s="7"/>
       <c r="N95" s="7"/>
     </row>
-    <row r="96" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B96" s="13"/>
+    <row r="96" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B96" s="29"/>
       <c r="C96" s="8" t="s">
         <v>83</v>
       </c>
@@ -3116,9 +3152,115 @@
       <c r="M96" s="7"/>
       <c r="N96" s="7"/>
     </row>
+    <row r="97" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B97" s="29"/>
+      <c r="C97" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="D97" s="7">
+        <v>1886</v>
+      </c>
+      <c r="E97" s="7"/>
+      <c r="F97" s="4"/>
+      <c r="G97" s="4"/>
+      <c r="H97" s="4"/>
+      <c r="I97" s="4"/>
+      <c r="J97" s="4"/>
+      <c r="K97" s="7">
+        <f>D97/2</f>
+        <v>943</v>
+      </c>
+      <c r="L97" s="7">
+        <f>D97/2</f>
+        <v>943</v>
+      </c>
+      <c r="M97" s="7"/>
+      <c r="N97" s="7"/>
+    </row>
+    <row r="98" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B98" s="29"/>
+      <c r="C98" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="D98" s="27">
+        <v>670</v>
+      </c>
+      <c r="E98" s="7"/>
+      <c r="F98" s="4"/>
+      <c r="G98" s="4"/>
+      <c r="H98" s="4"/>
+      <c r="I98" s="4"/>
+      <c r="J98" s="4"/>
+      <c r="K98" s="7">
+        <f>D98/2</f>
+        <v>335</v>
+      </c>
+      <c r="L98" s="7">
+        <f>D98/2</f>
+        <v>335</v>
+      </c>
+      <c r="M98" s="7"/>
+      <c r="N98" s="7"/>
+    </row>
+    <row r="99" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B99" s="29"/>
+      <c r="C99" s="26" t="s">
+        <v>92</v>
+      </c>
+      <c r="D99" s="27">
+        <v>580</v>
+      </c>
+      <c r="E99" s="7"/>
+      <c r="F99" s="4"/>
+      <c r="G99" s="4"/>
+      <c r="H99" s="4"/>
+      <c r="I99" s="4"/>
+      <c r="J99" s="4"/>
+      <c r="K99" s="7">
+        <f>D99/4</f>
+        <v>145</v>
+      </c>
+      <c r="L99" s="7">
+        <f>D99/4</f>
+        <v>145</v>
+      </c>
+      <c r="M99" s="7">
+        <f>D99/4</f>
+        <v>145</v>
+      </c>
+      <c r="N99" s="7">
+        <f>D99/4</f>
+        <v>145</v>
+      </c>
+    </row>
+    <row r="100" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B100" s="30"/>
+      <c r="C100" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D100" s="7">
+        <f>4490*2</f>
+        <v>8980</v>
+      </c>
+      <c r="E100" s="7"/>
+      <c r="F100" s="4"/>
+      <c r="G100" s="4"/>
+      <c r="H100" s="4"/>
+      <c r="I100" s="4"/>
+      <c r="J100" s="4"/>
+      <c r="K100" s="7">
+        <f>D100/2</f>
+        <v>4490</v>
+      </c>
+      <c r="L100" s="7">
+        <f>D100/2</f>
+        <v>4490</v>
+      </c>
+      <c r="M100" s="7"/>
+      <c r="N100" s="7"/>
+    </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B91:B96"/>
     <mergeCell ref="S8:S9"/>
     <mergeCell ref="S10:W10"/>
     <mergeCell ref="S13:W13"/>
@@ -3130,6 +3272,7 @@
     <mergeCell ref="B38:B39"/>
     <mergeCell ref="B40:B57"/>
     <mergeCell ref="B58:B64"/>
+    <mergeCell ref="B91:B100"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>

<commit_message>
Update Japan expense spreadsheet
</commit_message>
<xml_diff>
--- a/JAPAN EXPENSE.xlsx
+++ b/JAPAN EXPENSE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amadeusworkplace-my.sharepoint.com/personal/jonjester_reguyal_amadeus_com/Documents/Desktop/JAPAN TRIP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="368" documentId="8_{8DD0C82D-92A8-469F-8A5F-7373CA3C28E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0425E365-0358-4AA7-ACA8-DC7E48A7E1CC}"/>
+  <xr:revisionPtr revIDLastSave="375" documentId="8_{8DD0C82D-92A8-469F-8A5F-7373CA3C28E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76762EC0-90F8-4380-8FAE-CEE9AEEFA51A}"/>
   <bookViews>
     <workbookView xWindow="-30828" yWindow="-2916" windowWidth="30936" windowHeight="16776" xr2:uid="{77262E9F-01AC-4670-AAC1-0C05B2A698AE}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="95">
   <si>
     <t xml:space="preserve">FLIGHT </t>
   </si>
@@ -321,6 +321,9 @@
   </si>
   <si>
     <t>JAPAN VISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ClOTHES </t>
   </si>
 </sst>
 </file>
@@ -416,7 +419,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -502,23 +505,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -545,6 +537,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -585,20 +580,11 @@
     <xf numFmtId="17" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -939,7 +925,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{228C58C2-89C8-422F-BB16-5EF3E8507030}">
-  <dimension ref="B1:W100"/>
+  <dimension ref="B1:W101"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="8.85546875" style="11"/>
@@ -988,7 +974,7 @@
       </c>
     </row>
     <row r="2" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B2" s="21">
+      <c r="B2" s="22">
         <v>42491</v>
       </c>
       <c r="C2" s="4" t="s">
@@ -1013,7 +999,7 @@
       <c r="N2" s="7"/>
     </row>
     <row r="3" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B3" s="21"/>
+      <c r="B3" s="22"/>
       <c r="C3" s="8" t="s">
         <v>32</v>
       </c>
@@ -1035,7 +1021,7 @@
       <c r="N3" s="7"/>
     </row>
     <row r="4" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B4" s="21"/>
+      <c r="B4" s="22"/>
       <c r="C4" s="4" t="s">
         <v>7</v>
       </c>
@@ -1058,7 +1044,7 @@
       <c r="N4" s="7"/>
     </row>
     <row r="5" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B5" s="21"/>
+      <c r="B5" s="22"/>
       <c r="C5" s="8" t="s">
         <v>32</v>
       </c>
@@ -1081,7 +1067,7 @@
       <c r="N5" s="7"/>
     </row>
     <row r="6" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B6" s="21"/>
+      <c r="B6" s="22"/>
       <c r="C6" s="4" t="s">
         <v>6</v>
       </c>
@@ -1110,7 +1096,7 @@
       </c>
     </row>
     <row r="7" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B7" s="21"/>
+      <c r="B7" s="22"/>
       <c r="C7" s="8" t="s">
         <v>38</v>
       </c>
@@ -1133,7 +1119,7 @@
       <c r="N7" s="7"/>
     </row>
     <row r="8" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B8" s="21"/>
+      <c r="B8" s="22"/>
       <c r="C8" s="4" t="s">
         <v>5</v>
       </c>
@@ -1160,7 +1146,7 @@
         <f>D9/4</f>
         <v>1158</v>
       </c>
-      <c r="S8" s="13" t="s">
+      <c r="S8" s="14" t="s">
         <v>75</v>
       </c>
       <c r="T8" s="2" t="s">
@@ -1177,7 +1163,7 @@
       </c>
     </row>
     <row r="9" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B9" s="21"/>
+      <c r="B9" s="22"/>
       <c r="C9" s="8" t="s">
         <v>38</v>
       </c>
@@ -1198,10 +1184,10 @@
       <c r="L9" s="7"/>
       <c r="M9" s="7"/>
       <c r="N9" s="7"/>
-      <c r="S9" s="14"/>
+      <c r="S9" s="15"/>
       <c r="T9" s="3">
-        <f>SUM(K2:K100)</f>
-        <v>84847.909999999974</v>
+        <f>SUM(K2:K101)</f>
+        <v>92520.909999999974</v>
       </c>
       <c r="U9" s="3">
         <f>SUM(L2:L100)</f>
@@ -1211,7 +1197,7 @@
       <c r="W9" s="4"/>
     </row>
     <row r="10" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B10" s="21"/>
+      <c r="B10" s="22"/>
       <c r="C10" s="4" t="s">
         <v>8</v>
       </c>
@@ -1238,14 +1224,14 @@
         <f>D11/4</f>
         <v>256</v>
       </c>
-      <c r="S10" s="15"/>
-      <c r="T10" s="16"/>
-      <c r="U10" s="16"/>
-      <c r="V10" s="16"/>
-      <c r="W10" s="17"/>
+      <c r="S10" s="16"/>
+      <c r="T10" s="17"/>
+      <c r="U10" s="17"/>
+      <c r="V10" s="17"/>
+      <c r="W10" s="18"/>
     </row>
     <row r="11" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B11" s="21"/>
+      <c r="B11" s="22"/>
       <c r="C11" s="4"/>
       <c r="D11" s="7">
         <f>256*4</f>
@@ -1278,7 +1264,7 @@
       </c>
     </row>
     <row r="12" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B12" s="21"/>
+      <c r="B12" s="22"/>
       <c r="C12" s="4" t="s">
         <v>11</v>
       </c>
@@ -1321,7 +1307,7 @@
       </c>
     </row>
     <row r="13" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B13" s="21"/>
+      <c r="B13" s="22"/>
       <c r="C13" s="8" t="s">
         <v>32</v>
       </c>
@@ -1338,14 +1324,14 @@
       <c r="L13" s="7"/>
       <c r="M13" s="7"/>
       <c r="N13" s="7"/>
-      <c r="S13" s="15"/>
-      <c r="T13" s="16"/>
-      <c r="U13" s="16"/>
-      <c r="V13" s="16"/>
-      <c r="W13" s="17"/>
+      <c r="S13" s="16"/>
+      <c r="T13" s="17"/>
+      <c r="U13" s="17"/>
+      <c r="V13" s="17"/>
+      <c r="W13" s="18"/>
     </row>
     <row r="14" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B14" s="22">
+      <c r="B14" s="23">
         <v>42856</v>
       </c>
       <c r="C14" s="4" t="s">
@@ -1385,7 +1371,7 @@
       </c>
     </row>
     <row r="15" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B15" s="22"/>
+      <c r="B15" s="23"/>
       <c r="C15" s="8" t="s">
         <v>30</v>
       </c>
@@ -1421,7 +1407,7 @@
       <c r="W15" s="4"/>
     </row>
     <row r="16" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B16" s="22"/>
+      <c r="B16" s="23"/>
       <c r="C16" s="4" t="s">
         <v>12</v>
       </c>
@@ -1444,7 +1430,7 @@
       <c r="N16" s="7"/>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B17" s="22"/>
+      <c r="B17" s="23"/>
       <c r="C17" s="8" t="s">
         <v>36</v>
       </c>
@@ -1463,7 +1449,7 @@
       <c r="N17" s="7"/>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B18" s="22"/>
+      <c r="B18" s="23"/>
       <c r="C18" s="8" t="s">
         <v>37</v>
       </c>
@@ -1482,7 +1468,7 @@
       <c r="N18" s="7"/>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B19" s="22"/>
+      <c r="B19" s="23"/>
       <c r="C19" s="4" t="s">
         <v>13</v>
       </c>
@@ -1502,7 +1488,7 @@
       <c r="N19" s="7"/>
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B20" s="22"/>
+      <c r="B20" s="23"/>
       <c r="C20" s="8" t="s">
         <v>35</v>
       </c>
@@ -1521,7 +1507,7 @@
       <c r="N20" s="7"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B21" s="22"/>
+      <c r="B21" s="23"/>
       <c r="C21" s="4" t="s">
         <v>14</v>
       </c>
@@ -1544,7 +1530,7 @@
       <c r="N21" s="7"/>
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B22" s="22"/>
+      <c r="B22" s="23"/>
       <c r="C22" s="8" t="s">
         <v>89</v>
       </c>
@@ -1564,7 +1550,7 @@
       <c r="N22" s="7"/>
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B23" s="22"/>
+      <c r="B23" s="23"/>
       <c r="C23" s="8" t="s">
         <v>34</v>
       </c>
@@ -1587,7 +1573,7 @@
       <c r="N23" s="7"/>
     </row>
     <row r="24" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B24" s="22"/>
+      <c r="B24" s="23"/>
       <c r="C24" s="4" t="s">
         <v>15</v>
       </c>
@@ -1607,7 +1593,7 @@
       <c r="N24" s="7"/>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B25" s="22"/>
+      <c r="B25" s="23"/>
       <c r="C25" s="8" t="s">
         <v>33</v>
       </c>
@@ -1626,7 +1612,7 @@
       <c r="N25" s="7"/>
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B26" s="22"/>
+      <c r="B26" s="23"/>
       <c r="C26" s="4" t="s">
         <v>16</v>
       </c>
@@ -1649,7 +1635,7 @@
       <c r="N26" s="7"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B27" s="22"/>
+      <c r="B27" s="23"/>
       <c r="C27" s="8" t="s">
         <v>30</v>
       </c>
@@ -1668,7 +1654,7 @@
       <c r="N27" s="7"/>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B28" s="22"/>
+      <c r="B28" s="23"/>
       <c r="C28" s="8" t="s">
         <v>31</v>
       </c>
@@ -1687,7 +1673,7 @@
       <c r="N28" s="7"/>
     </row>
     <row r="29" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B29" s="22"/>
+      <c r="B29" s="23"/>
       <c r="C29" s="4" t="s">
         <v>17</v>
       </c>
@@ -1710,7 +1696,7 @@
       <c r="N29" s="7"/>
     </row>
     <row r="30" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B30" s="22"/>
+      <c r="B30" s="23"/>
       <c r="C30" s="8" t="s">
         <v>32</v>
       </c>
@@ -1729,7 +1715,7 @@
       <c r="N30" s="7"/>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B31" s="22"/>
+      <c r="B31" s="23"/>
       <c r="C31" s="4" t="s">
         <v>18</v>
       </c>
@@ -1752,7 +1738,7 @@
       <c r="N31" s="7"/>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B32" s="22"/>
+      <c r="B32" s="23"/>
       <c r="C32" s="8" t="s">
         <v>30</v>
       </c>
@@ -1772,7 +1758,7 @@
       <c r="N32" s="7"/>
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B33" s="22"/>
+      <c r="B33" s="23"/>
       <c r="C33" s="8" t="s">
         <v>31</v>
       </c>
@@ -1795,7 +1781,7 @@
       <c r="N33" s="7"/>
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B34" s="22"/>
+      <c r="B34" s="23"/>
       <c r="C34" s="4" t="s">
         <v>19</v>
       </c>
@@ -1821,7 +1807,7 @@
       </c>
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B35" s="22"/>
+      <c r="B35" s="23"/>
       <c r="C35" s="8" t="s">
         <v>27</v>
       </c>
@@ -1841,7 +1827,7 @@
       <c r="N35" s="7"/>
     </row>
     <row r="36" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B36" s="22"/>
+      <c r="B36" s="23"/>
       <c r="C36" s="8" t="s">
         <v>28</v>
       </c>
@@ -1861,7 +1847,7 @@
       <c r="N36" s="7"/>
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B37" s="22"/>
+      <c r="B37" s="23"/>
       <c r="C37" s="8" t="s">
         <v>29</v>
       </c>
@@ -1883,7 +1869,7 @@
       <c r="N37" s="7"/>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B38" s="23">
+      <c r="B38" s="24">
         <v>43221</v>
       </c>
       <c r="C38" s="4" t="s">
@@ -1908,7 +1894,7 @@
       <c r="N38" s="7"/>
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B39" s="23"/>
+      <c r="B39" s="24"/>
       <c r="C39" s="8" t="s">
         <v>87</v>
       </c>
@@ -1927,7 +1913,7 @@
       <c r="N39" s="7"/>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B40" s="24">
+      <c r="B40" s="25">
         <v>43586</v>
       </c>
       <c r="C40" s="4" t="s">
@@ -1949,7 +1935,7 @@
       <c r="N40" s="7"/>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B41" s="24"/>
+      <c r="B41" s="25"/>
       <c r="C41" s="8" t="s">
         <v>88</v>
       </c>
@@ -1968,7 +1954,7 @@
       <c r="N41" s="7"/>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B42" s="24"/>
+      <c r="B42" s="25"/>
       <c r="C42" s="4" t="s">
         <v>22</v>
       </c>
@@ -1994,7 +1980,7 @@
       </c>
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B43" s="24"/>
+      <c r="B43" s="25"/>
       <c r="C43" s="8" t="s">
         <v>26</v>
       </c>
@@ -2013,7 +1999,7 @@
       <c r="N43" s="7"/>
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B44" s="24"/>
+      <c r="B44" s="25"/>
       <c r="C44" s="8" t="s">
         <v>1</v>
       </c>
@@ -2032,7 +2018,7 @@
       <c r="N44" s="7"/>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B45" s="24"/>
+      <c r="B45" s="25"/>
       <c r="C45" s="8" t="s">
         <v>4</v>
       </c>
@@ -2051,7 +2037,7 @@
       <c r="N45" s="7"/>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B46" s="24"/>
+      <c r="B46" s="25"/>
       <c r="C46" s="4" t="s">
         <v>23</v>
       </c>
@@ -2074,7 +2060,7 @@
       <c r="N46" s="7"/>
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B47" s="24"/>
+      <c r="B47" s="25"/>
       <c r="C47" s="8" t="s">
         <v>39</v>
       </c>
@@ -2093,7 +2079,7 @@
       <c r="N47" s="7"/>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B48" s="24"/>
+      <c r="B48" s="25"/>
       <c r="C48" s="4" t="s">
         <v>24</v>
       </c>
@@ -2110,7 +2096,7 @@
       <c r="N48" s="7"/>
     </row>
     <row r="49" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B49" s="24"/>
+      <c r="B49" s="25"/>
       <c r="C49" s="8" t="s">
         <v>40</v>
       </c>
@@ -2142,7 +2128,7 @@
       </c>
     </row>
     <row r="50" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B50" s="24"/>
+      <c r="B50" s="25"/>
       <c r="C50" s="8" t="s">
         <v>42</v>
       </c>
@@ -2162,7 +2148,7 @@
       <c r="N50" s="7"/>
     </row>
     <row r="51" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B51" s="24"/>
+      <c r="B51" s="25"/>
       <c r="C51" s="8" t="s">
         <v>41</v>
       </c>
@@ -2182,7 +2168,7 @@
       <c r="N51" s="7"/>
     </row>
     <row r="52" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B52" s="24"/>
+      <c r="B52" s="25"/>
       <c r="C52" s="8" t="s">
         <v>43</v>
       </c>
@@ -2205,7 +2191,7 @@
       <c r="N52" s="7"/>
     </row>
     <row r="53" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B53" s="24"/>
+      <c r="B53" s="25"/>
       <c r="C53" s="4" t="s">
         <v>25</v>
       </c>
@@ -2225,7 +2211,7 @@
       <c r="N53" s="7"/>
     </row>
     <row r="54" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B54" s="24"/>
+      <c r="B54" s="25"/>
       <c r="C54" s="8" t="s">
         <v>44</v>
       </c>
@@ -2244,7 +2230,7 @@
       <c r="N54" s="7"/>
     </row>
     <row r="55" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B55" s="24"/>
+      <c r="B55" s="25"/>
       <c r="C55" s="9" t="s">
         <v>45</v>
       </c>
@@ -2267,7 +2253,7 @@
       <c r="N55" s="7"/>
     </row>
     <row r="56" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B56" s="24"/>
+      <c r="B56" s="25"/>
       <c r="C56" s="8" t="s">
         <v>2</v>
       </c>
@@ -2286,7 +2272,7 @@
       <c r="N56" s="7"/>
     </row>
     <row r="57" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B57" s="24"/>
+      <c r="B57" s="25"/>
       <c r="C57" s="8" t="s">
         <v>1</v>
       </c>
@@ -2307,7 +2293,7 @@
       <c r="N57" s="7"/>
     </row>
     <row r="58" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B58" s="25">
+      <c r="B58" s="26">
         <v>43952</v>
       </c>
       <c r="C58" s="9" t="s">
@@ -2329,7 +2315,7 @@
       <c r="N58" s="7"/>
     </row>
     <row r="59" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B59" s="25"/>
+      <c r="B59" s="26"/>
       <c r="C59" s="8" t="s">
         <v>48</v>
       </c>
@@ -2348,7 +2334,7 @@
       <c r="N59" s="7"/>
     </row>
     <row r="60" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B60" s="25"/>
+      <c r="B60" s="26"/>
       <c r="C60" s="9" t="s">
         <v>49</v>
       </c>
@@ -2371,7 +2357,7 @@
       <c r="N60" s="7"/>
     </row>
     <row r="61" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B61" s="25"/>
+      <c r="B61" s="26"/>
       <c r="C61" s="8" t="s">
         <v>50</v>
       </c>
@@ -2390,7 +2376,7 @@
       <c r="N61" s="7"/>
     </row>
     <row r="62" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B62" s="25"/>
+      <c r="B62" s="26"/>
       <c r="C62" s="9" t="s">
         <v>51</v>
       </c>
@@ -2413,7 +2399,7 @@
       <c r="N62" s="7"/>
     </row>
     <row r="63" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B63" s="25"/>
+      <c r="B63" s="26"/>
       <c r="C63" s="8" t="s">
         <v>52</v>
       </c>
@@ -2433,7 +2419,7 @@
       <c r="N63" s="7"/>
     </row>
     <row r="64" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B64" s="25"/>
+      <c r="B64" s="26"/>
       <c r="C64" s="8" t="s">
         <v>53</v>
       </c>
@@ -2455,7 +2441,7 @@
       <c r="N64" s="7"/>
     </row>
     <row r="65" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B65" s="18">
+      <c r="B65" s="19">
         <v>44317</v>
       </c>
       <c r="C65" s="9" t="s">
@@ -2477,7 +2463,7 @@
       <c r="N65" s="7"/>
     </row>
     <row r="66" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B66" s="18"/>
+      <c r="B66" s="19"/>
       <c r="C66" s="8" t="s">
         <v>55</v>
       </c>
@@ -2496,7 +2482,7 @@
       <c r="N66" s="7"/>
     </row>
     <row r="67" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B67" s="18"/>
+      <c r="B67" s="19"/>
       <c r="C67" s="9" t="s">
         <v>10</v>
       </c>
@@ -2522,7 +2508,7 @@
       <c r="N67" s="7"/>
     </row>
     <row r="68" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B68" s="18"/>
+      <c r="B68" s="19"/>
       <c r="C68" s="8" t="s">
         <v>56</v>
       </c>
@@ -2541,7 +2527,7 @@
       <c r="N68" s="7"/>
     </row>
     <row r="69" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B69" s="19">
+      <c r="B69" s="20">
         <v>44682</v>
       </c>
       <c r="C69" s="9" t="s">
@@ -2566,7 +2552,7 @@
       <c r="N69" s="7"/>
     </row>
     <row r="70" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B70" s="19"/>
+      <c r="B70" s="20"/>
       <c r="C70" s="8" t="s">
         <v>58</v>
       </c>
@@ -2586,7 +2572,7 @@
       <c r="N70" s="7"/>
     </row>
     <row r="71" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B71" s="19"/>
+      <c r="B71" s="20"/>
       <c r="C71" s="8" t="s">
         <v>59</v>
       </c>
@@ -2608,7 +2594,7 @@
       <c r="N71" s="7"/>
     </row>
     <row r="72" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B72" s="19"/>
+      <c r="B72" s="20"/>
       <c r="C72" s="9" t="s">
         <v>60</v>
       </c>
@@ -2631,7 +2617,7 @@
       <c r="N72" s="7"/>
     </row>
     <row r="73" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B73" s="19"/>
+      <c r="B73" s="20"/>
       <c r="C73" s="8" t="s">
         <v>61</v>
       </c>
@@ -2650,7 +2636,7 @@
       <c r="N73" s="7"/>
     </row>
     <row r="74" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B74" s="19"/>
+      <c r="B74" s="20"/>
       <c r="C74" s="8" t="s">
         <v>62</v>
       </c>
@@ -2672,7 +2658,7 @@
       <c r="N74" s="7"/>
     </row>
     <row r="75" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B75" s="19"/>
+      <c r="B75" s="20"/>
       <c r="C75" s="8" t="s">
         <v>63</v>
       </c>
@@ -2695,7 +2681,7 @@
       <c r="N75" s="7"/>
     </row>
     <row r="76" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B76" s="19"/>
+      <c r="B76" s="20"/>
       <c r="C76" s="8" t="s">
         <v>64</v>
       </c>
@@ -2717,7 +2703,7 @@
       <c r="N76" s="7"/>
     </row>
     <row r="77" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B77" s="19"/>
+      <c r="B77" s="20"/>
       <c r="C77" s="9" t="s">
         <v>65</v>
       </c>
@@ -2737,7 +2723,7 @@
       <c r="N77" s="7"/>
     </row>
     <row r="78" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B78" s="19"/>
+      <c r="B78" s="20"/>
       <c r="C78" s="8" t="s">
         <v>66</v>
       </c>
@@ -2759,7 +2745,7 @@
       <c r="N78" s="7"/>
     </row>
     <row r="79" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B79" s="20">
+      <c r="B79" s="21">
         <v>45047</v>
       </c>
       <c r="C79" s="9" t="s">
@@ -2784,7 +2770,7 @@
       <c r="N79" s="7"/>
     </row>
     <row r="80" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B80" s="20"/>
+      <c r="B80" s="21"/>
       <c r="C80" s="8" t="s">
         <v>68</v>
       </c>
@@ -2804,7 +2790,7 @@
       <c r="N80" s="7"/>
     </row>
     <row r="81" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B81" s="20"/>
+      <c r="B81" s="21"/>
       <c r="C81" s="8" t="s">
         <v>69</v>
       </c>
@@ -2824,7 +2810,7 @@
       <c r="N81" s="7"/>
     </row>
     <row r="82" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B82" s="20"/>
+      <c r="B82" s="21"/>
       <c r="C82" s="8" t="s">
         <v>70</v>
       </c>
@@ -2847,7 +2833,7 @@
       <c r="N82" s="7"/>
     </row>
     <row r="83" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B83" s="20"/>
+      <c r="B83" s="21"/>
       <c r="C83" s="4"/>
       <c r="D83" s="7"/>
       <c r="E83" s="7"/>
@@ -2862,7 +2848,7 @@
       <c r="N83" s="7"/>
     </row>
     <row r="84" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B84" s="20"/>
+      <c r="B84" s="21"/>
       <c r="C84" s="9" t="s">
         <v>71</v>
       </c>
@@ -2885,7 +2871,7 @@
       <c r="N84" s="7"/>
     </row>
     <row r="85" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B85" s="20"/>
+      <c r="B85" s="21"/>
       <c r="C85" s="8" t="s">
         <v>32</v>
       </c>
@@ -2907,7 +2893,7 @@
       <c r="N85" s="7"/>
     </row>
     <row r="86" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B86" s="20"/>
+      <c r="B86" s="21"/>
       <c r="C86" s="9" t="s">
         <v>72</v>
       </c>
@@ -2930,7 +2916,7 @@
       <c r="N86" s="7"/>
     </row>
     <row r="87" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B87" s="20"/>
+      <c r="B87" s="21"/>
       <c r="C87" s="8" t="s">
         <v>32</v>
       </c>
@@ -2952,7 +2938,7 @@
       <c r="N87" s="7"/>
     </row>
     <row r="88" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B88" s="20"/>
+      <c r="B88" s="21"/>
       <c r="C88" s="4" t="s">
         <v>73</v>
       </c>
@@ -2975,7 +2961,7 @@
       <c r="N88" s="7"/>
     </row>
     <row r="89" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B89" s="20"/>
+      <c r="B89" s="21"/>
       <c r="C89" s="8" t="s">
         <v>69</v>
       </c>
@@ -2994,7 +2980,7 @@
       <c r="N89" s="7"/>
     </row>
     <row r="90" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B90" s="20"/>
+      <c r="B90" s="21"/>
       <c r="C90" s="8" t="s">
         <v>74</v>
       </c>
@@ -3016,7 +3002,7 @@
       <c r="N90" s="7"/>
     </row>
     <row r="91" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B91" s="28" t="s">
+      <c r="B91" s="27" t="s">
         <v>81</v>
       </c>
       <c r="C91" s="9" t="s">
@@ -3044,7 +3030,7 @@
       <c r="N91" s="7"/>
     </row>
     <row r="92" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B92" s="29"/>
+      <c r="B92" s="27"/>
       <c r="C92" s="8" t="s">
         <v>83</v>
       </c>
@@ -3063,7 +3049,7 @@
       <c r="N92" s="7"/>
     </row>
     <row r="93" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B93" s="29"/>
+      <c r="B93" s="27"/>
       <c r="C93" s="9" t="s">
         <v>84</v>
       </c>
@@ -3089,7 +3075,7 @@
       <c r="N93" s="7"/>
     </row>
     <row r="94" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B94" s="29"/>
+      <c r="B94" s="27"/>
       <c r="C94" s="8" t="s">
         <v>83</v>
       </c>
@@ -3108,7 +3094,7 @@
       <c r="N94" s="7"/>
     </row>
     <row r="95" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B95" s="29"/>
+      <c r="B95" s="27"/>
       <c r="C95" s="9" t="s">
         <v>85</v>
       </c>
@@ -3134,7 +3120,7 @@
       <c r="N95" s="7"/>
     </row>
     <row r="96" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B96" s="29"/>
+      <c r="B96" s="27"/>
       <c r="C96" s="8" t="s">
         <v>83</v>
       </c>
@@ -3153,8 +3139,8 @@
       <c r="N96" s="7"/>
     </row>
     <row r="97" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B97" s="29"/>
-      <c r="C97" s="26" t="s">
+      <c r="B97" s="27"/>
+      <c r="C97" s="9" t="s">
         <v>90</v>
       </c>
       <c r="D97" s="7">
@@ -3178,11 +3164,11 @@
       <c r="N97" s="7"/>
     </row>
     <row r="98" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B98" s="29"/>
-      <c r="C98" s="26" t="s">
+      <c r="B98" s="27"/>
+      <c r="C98" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="D98" s="27">
+      <c r="D98" s="13">
         <v>670</v>
       </c>
       <c r="E98" s="7"/>
@@ -3203,11 +3189,11 @@
       <c r="N98" s="7"/>
     </row>
     <row r="99" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B99" s="29"/>
-      <c r="C99" s="26" t="s">
+      <c r="B99" s="27"/>
+      <c r="C99" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="D99" s="27">
+      <c r="D99" s="13">
         <v>580</v>
       </c>
       <c r="E99" s="7"/>
@@ -3234,7 +3220,7 @@
       </c>
     </row>
     <row r="100" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B100" s="30"/>
+      <c r="B100" s="27"/>
       <c r="C100" s="4" t="s">
         <v>93</v>
       </c>
@@ -3259,20 +3245,42 @@
       <c r="M100" s="7"/>
       <c r="N100" s="7"/>
     </row>
+    <row r="101" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B101" s="27"/>
+      <c r="C101" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="D101" s="7">
+        <v>7673</v>
+      </c>
+      <c r="E101" s="7"/>
+      <c r="F101" s="4"/>
+      <c r="G101" s="4"/>
+      <c r="H101" s="4"/>
+      <c r="I101" s="4"/>
+      <c r="J101" s="4"/>
+      <c r="K101" s="7">
+        <f>D101</f>
+        <v>7673</v>
+      </c>
+      <c r="L101" s="7"/>
+      <c r="M101" s="7"/>
+      <c r="N101" s="7"/>
+    </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="S8:S9"/>
-    <mergeCell ref="S10:W10"/>
-    <mergeCell ref="S13:W13"/>
-    <mergeCell ref="B65:B68"/>
-    <mergeCell ref="B69:B78"/>
+    <mergeCell ref="B91:B101"/>
     <mergeCell ref="B79:B90"/>
     <mergeCell ref="B2:B13"/>
     <mergeCell ref="B14:B37"/>
     <mergeCell ref="B38:B39"/>
     <mergeCell ref="B40:B57"/>
     <mergeCell ref="B58:B64"/>
-    <mergeCell ref="B91:B100"/>
+    <mergeCell ref="S8:S9"/>
+    <mergeCell ref="S10:W10"/>
+    <mergeCell ref="S13:W13"/>
+    <mergeCell ref="B65:B68"/>
+    <mergeCell ref="B69:B78"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter>

</xml_diff>